<commit_message>
push module 04: static testing
</commit_message>
<xml_diff>
--- a/module03-white-box-technique/03_44_NguyenVanMinh_Module03.xlsx
+++ b/module03-white-box-technique/03_44_NguyenVanMinh_Module03.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\University\2025_HK1\DamBaoChatLuongVaKiemThuPhanMem\github\module03-white-box-technique\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE524D99-3CDF-4A9C-93A2-F03FFB0FD2AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C26DA02-C535-4628-A4E6-CDFC71149564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="7" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="7" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Result" sheetId="22" r:id="rId1"/>
@@ -6881,6 +6881,526 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>213480</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>115061</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>309600</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>10926</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="50" name="Ink 49">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B1BF671-7C8D-2515-D3B3-4B4610F81224}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="213480" y="849651"/>
+            <a:ext cx="96120" cy="263160"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="50" name="Ink 49">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B1BF671-7C8D-2515-D3B3-4B4610F81224}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="207360" y="843531"/>
+              <a:ext cx="108360" cy="275400"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>180000</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>122166</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>82336</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>21849</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="57" name="Ink 56">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4965200-8F5B-2584-79D3-503ADA922240}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="180000" y="1224051"/>
+            <a:ext cx="510840" cy="817920"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="57" name="Ink 56">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4965200-8F5B-2584-79D3-503ADA922240}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="173880" y="1217931"/>
+              <a:ext cx="523080" cy="830160"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>116536</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>122934</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>388503</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>101911</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="63" name="Ink 62">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A782A730-B85B-7697-9061-6B678FA50052}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="725040" y="2143056"/>
+            <a:ext cx="417240" cy="529920"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="63" name="Ink 62">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A782A730-B85B-7697-9061-6B678FA50052}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="718920" y="2136936"/>
+              <a:ext cx="429480" cy="542160"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>39303</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>147224</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>234783</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>100016</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="68" name="Ink 67">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{246E1671-90FE-D060-FBF0-819BDA0F0798}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="793080" y="2901936"/>
+            <a:ext cx="195480" cy="136440"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="68" name="Ink 67">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{246E1671-90FE-D060-FBF0-819BDA0F0798}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="786949" y="2895800"/>
+              <a:ext cx="207743" cy="148712"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>462600</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>133951</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>524520</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>114104</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="69" name="Ink 68">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE183769-BDBE-B4E4-0FAA-6FF447DFFEAB}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="462600" y="2705016"/>
+            <a:ext cx="61920" cy="163800"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="69" name="Ink 68">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE183769-BDBE-B4E4-0FAA-6FF447DFFEAB}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="456444" y="2698883"/>
+              <a:ext cx="74232" cy="176067"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>202320</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>164096</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>347400</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>92769</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="72" name="Ink 71">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1CB6A64-70F5-C7EC-8447-BCF3312084E4}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="202320" y="3102456"/>
+            <a:ext cx="145080" cy="112320"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="72" name="Ink 71">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1CB6A64-70F5-C7EC-8447-BCF3312084E4}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="196200" y="3096336"/>
+              <a:ext cx="157320" cy="124560"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>408240</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>5241</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>52096</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>128361</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="76" name="Ink 75">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E00C316A-3C55-D1D2-96F6-E438C2FF32AF}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="408240" y="3310896"/>
+            <a:ext cx="252360" cy="123120"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="76" name="Ink 75">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E00C316A-3C55-D1D2-96F6-E438C2FF32AF}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="402120" y="3304776"/>
+              <a:ext cx="264600" cy="135360"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>60120</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>172320</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>208440</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>161833</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="81" name="Ink 80">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{019485B0-61BA-A6E9-D7AE-2DB884EE6D26}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="60120" y="3477975"/>
+            <a:ext cx="148320" cy="173160"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="81" name="Ink 80">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{019485B0-61BA-A6E9-D7AE-2DB884EE6D26}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="53985" y="3471868"/>
+              <a:ext cx="160590" cy="185375"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -11754,6 +12274,235 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:54.858"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">332 96 24575,'1'-1'0,"0"-1"0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,4-1 0,13-7 0,-11 3 0,1-1 0,0 0 0,0 0 0,1 1 0,0 0 0,0 1 0,0 0 0,1 0 0,-1 1 0,19-3 0,22 1 0,0 2 0,0 3 0,60 6 0,-108-6 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,3 3 0,-3-4 0,-1 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-2 4 0,-1 3 0,-1 0 0,-1-1 0,0 1 0,0-1 0,-1 0 0,0 0 0,0-1 0,-14 14 0,3-8 0,0 0 0,-1-1 0,0 0 0,-37 16 0,5-2 0,4 5 0,38-24 0,0-1 0,-1 0 0,0-1 0,0 0 0,-19 8 0,9-6 0,0 0 0,1 1 0,0 1 0,0 0 0,1 2 0,-27 20 0,-11 5 0,42-29 0,0 1 0,1 0 0,-16 14 0,16-10 0,-1-1 0,-1 0 0,0 0 0,0-1 0,-1-1 0,-1 0 0,-16 6 0,26-12 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,1 1 0,0-1 0,0 1 0,0 0 0,1 0 0,0 0 0,-5 7 0,8-10 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,2 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,0 3 0,0-3 0,1 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,1-1 0,0 0 0,2 2 0,26 7 0,0-1 0,0-1 0,0-2 0,1-1 0,0-1 0,0-1 0,44-3 0,81 10 0,76 32 0,-193-38 0,1-1 0,0-2 0,40-4 0,-43 0 0,0 2 0,0 2 0,59 8 0,-93-8 0,1-1 0,-1 1 0,1 1 0,-1-1 0,1 0 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,-3 8 0,2-8 0,0-1 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,1-1 0,-2 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,-6 1 0,-60 16 0,48-15 0,-30 7 0,30-8 0,1 1 0,0 1 0,-36 14 0,17 3 0,30-16 0,1-1 0,-1 0 0,0 0 0,-16 5 0,-44 15 78,51-17-559,-1 0 0,-32 7 0,29-11-6345</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink101.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:58.689"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1221 1 24575,'-13'0'0,"0"0"0,-1 2 0,1 0 0,0 0 0,0 1 0,0 1 0,1 0 0,-1 0 0,1 2 0,0-1 0,0 2 0,1-1 0,0 1 0,0 1 0,0 0 0,1 1 0,-10 11 0,-1 3 0,1 0 0,1 2 0,1 0 0,2 1 0,-16 31 0,-8 19 0,30-61 0,0 1 0,2 0 0,0 1 0,1 0 0,0 0 0,2 1 0,0 0 0,1 0 0,-3 29 0,3-7 0,-1 0 0,-2-1 0,-14 45 0,11-42 0,1 7 0,3 0 0,2 0 0,2 0 0,7 68 0,-2 0 0,-2-106 0,0 0 0,1 1 0,0-1 0,1-1 0,0 1 0,1 0 0,0-1 0,0 1 0,1-1 0,1-1 0,0 1 0,0-1 0,1 0 0,0 0 0,1 0 0,12 10 0,58 32 0,-70-46 0,0 1 0,1-1 0,-1 0 0,1-1 0,0 1 0,1-2 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0-1 0,0 0 0,0 0 0,0 0 0,12-2 0,-13 0 0,-1 1 0,1-1 0,0 0 0,-1-1 0,1 0 0,-1-1 0,0 1 0,0-1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 0 0,0-1 0,-1 1 0,8-10 0,25-30 0,-31 37 0,0 0 0,0-1 0,-1 0 0,0-1 0,-1 0 0,0 0 0,0 0 0,-1-1 0,6-17 0,-9 17 0,1 0 0,1 0 0,0 0 0,0 0 0,1 1 0,0 0 0,1 0 0,0 0 0,1 1 0,0 0 0,0 0 0,1 0 0,15-12 0,-14 13 0,-1 0 0,0-1 0,-1-1 0,0 1 0,0-1 0,-1 0 0,0-1 0,0 1 0,-2-1 0,1 0 0,-1-1 0,-1 1 0,3-13 0,-2-1 0,0 0 0,-2 0 0,-1 0 0,0 0 0,-5-30 0,3 51 0,0 0 0,0 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,-1 0 0,1 1 0,-6-5 0,3 3 0,0 0 0,1-1 0,0 0 0,0-1 0,-6-7 0,3 2 0,-1 1 0,0 1 0,0-1 0,-1 1 0,0 1 0,-15-10 0,11 8 0,1 0 0,0-1 0,-13-14 0,22 20 0,-1 1 0,0 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 1 0,-1-1 0,1 1 0,-8 0 0,-15-1 0,0 1 0,-35 4 0,13 0 0,30-4 0,0 2 0,0 0 0,1 2 0,-1 0 0,0 1 0,1 1 0,-27 10 0,21-5 0,-44 9 0,55-16 0,0 1 0,0 0 0,0 1 0,0 0 0,1 1 0,0 1 0,0 0 0,-21 15 0,19-9 0,-1-1 0,0-1 0,-1-1 0,-27 11 0,25-9 0,0 0 0,0 1 0,2 1 0,-27 25 0,13-11 0,-78 74 0,100-92 17,0 1-1,0 0 1,0 0 0,2 1-1,-1 0 1,2 1-1,-11 21 1,10-17-392,-2 0 1,0 0-1,-17 20 1,15-23-6452</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink102.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:57.160"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">103 3 24575,'1'69'0,"-3"80"0,0-137 0,-1 0 0,0 0 0,-1 0 0,0 0 0,-1-1 0,-7 13 0,-17 44 0,21-42 0,-2 8 0,-9 53 0,18-78 0,0 1 0,0-1 0,1 1 0,1-1 0,-1 1 0,1 0 0,1-1 0,0 0 0,1 1 0,5 13 0,-4-17 0,0-1 0,1 1 0,-1-1 0,1 0 0,1 0 0,-1 0 0,1-1 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,1-2 0,11 4 0,33 19 0,-18-7 0,0-1 0,1-2 0,1-1 0,36 10 0,-44-15 0,-21-7 0,-1 0 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 1 0,1 0 0,-1 0 0,0 0 0,4 6 0,36 58 0,-23-32 0,-13-21 0,0 0 0,-1 0 0,-1 1 0,6 26 0,-6-22 0,0-1 0,15 32 0,-11-29 0,-1 0 0,-1 0 0,9 38 0,-16-57 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,-2 3 0,0-2 0,0-1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,-1 1 0,0-1 0,0 0 0,0-1 0,-8 3 0,-13 0 0,1-1 0,-1-1 0,1-1 0,-30-2 0,46 1 0,-33-1 0,29 2 0,0 0 0,1-2 0,-1 1 0,0-2 0,0 1 0,0-2 0,1 1 0,0-2 0,-18-6 0,11 0 40,1 0 0,-23-17 0,35 22-175,0 1 0,1-1 0,0-1 0,0 1 0,0-1 0,1 0 0,0 0 0,0 0 0,1 0 0,-4-9 0,-1-6-6691</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="419.51">48 34 24575,'5'-3'0,"-1"0"0,1 0 0,0 0 0,0 0 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 1 0,-1 0 0,9-1 0,76-1 0,-61 3 0,50-2 0,239 6 0,-306-2 0,0 1 0,0 0 0,0 0 0,-1 1 0,0 1 0,16 7 0,41 16 0,-55-24 30,0 0-1,-1 2 0,19 9 1,11 6-1513,-22-14-5343</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink103.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:55.603"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">325 0 24575,'0'9'0,"-1"1"0,-1-1 0,1 0 0,-1 0 0,-1 0 0,1 0 0,-1-1 0,-1 1 0,0-1 0,-7 12 0,-7 9 0,-34 41 0,34-50 0,2 2 0,-25 44 0,32-47 0,2 1 0,-7 25 0,-13 36 0,17-57 0,-11 45 0,15-48 0,0 0 0,-2-1 0,-11 26 0,16-40 0,0 0 0,0 0 0,1 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,1 0 0,-1 0 0,1 0 0,1 0 0,-1 0 0,1 0 0,2 8 0,-2-10 0,0-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,0-1 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,8 2 0,25 1 0,1-1 0,-1-2 0,55-6 0,5 1 0,-59 5 0,-27 0 0,1 0 0,-1-1 0,0 0 0,0-1 0,1-1 0,-1 1 0,0-2 0,0 0 0,-1 0 0,12-5 0,45-32-1365,-50 26-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="446.47">520 535 24575,'-1'34'0,"-3"1"0,-7 37 0,5-37 0,-4 70 0,10-103 0,0 35 0,-1 0 0,-2-1 0,-10 53 0,7-50 0,1 1 0,2 1 0,2-1 0,4 50 0,-1-33 0,-4 58 0,-15-40-1365,11-54-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink104.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:25:03.802"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">692 1 24575,'-65'-1'0,"-77"3"0,137-1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,1 1 0,-5 4 0,-3 6 0,0 1 0,-17 29 0,-15 21 0,32-52 0,1 0 0,0 1 0,0 1 0,2-1 0,-1 2 0,2-1 0,0 1 0,-8 28 0,9-18 0,1 1 0,1 0 0,1 0 0,1 49 0,2 33 0,3 89 0,-2-190 0,0 0 0,1-1 0,0 1 0,0 0 0,1 0 0,0-1 0,0 0 0,1 1 0,0-1 0,0-1 0,10 13 0,3 0 0,1-1 0,27 22 0,-28-25 0,-9-7 0,0 0 0,-1 0 0,11 17 0,-14-18 0,1-1 0,0 1 0,0-1 0,0 0 0,1 0 0,0-1 0,0 1 0,0-1 0,9 4 0,1 1 0,-1 0 0,22 20 0,-6-5 0,-31-25 0,1 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,-16 5 0,-32-5 0,42-1 0,-10-2 0,0 0 0,0-2 0,0 0 0,0-1 0,1 0 0,-1-1 0,1-1 0,-19-12 0,-29-12 0,-121-37 0,178 66 0,1-1 0,0 1 0,1-1 0,-1-1 0,0 1 0,1-1 0,-1 0 0,1 0 0,0 0 0,1 0 0,-1-1 0,1 0 0,0 1 0,0-2 0,0 1 0,0 0 0,1 0 0,0-1 0,-1-5 0,0 3 0,1 0 0,-1 0 0,2 0 0,-1 0 0,1 0 0,1-1 0,-1 1 0,1 0 0,1 0 0,0-1 0,0 1 0,4-16 0,-4 21 0,1-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,6-3 0,3 1 0,-1 0 0,1 1 0,22-3 0,-25 4 0,1 1 0,0-1 0,0-1 0,-1 0 0,1 0 0,10-6 0,42-28 0,87-39 0,-137 70 0,-1 0 0,0-1 0,15-11 0,-18 11 0,1 1 0,0 0 0,0 1 0,0 0 0,20-7 0,-18 9 0,-1 0 0,1-1 0,-1 0 0,0 0 0,-1-1 0,1 0 0,-1-1 0,0 0 0,0 0 0,11-12 0,0-2 0,-12 14 0,-1-1 0,0 0 0,0-1 0,-1 1 0,0-1 0,8-14 0,-13 19 0,0 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,-3-4 0,-27-32-1365,18 22-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink105.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:25:02.154"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">567 1 24575,'-1'0'0,"0"0"0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,1-1 0,0 2 0,0 1 0,1 1 0,0 0 0,-1-1 0,1 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,3 3 0,0-2 0,1 0 0,0 0 0,-1-1 0,1 0 0,1 0 0,-1 0 0,0-1 0,1-1 0,13 3 0,73-1 0,-76-4 0,0 1 0,0 0 0,0 2 0,34 6 0,-52-8 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,-22 25 0,-38 16 0,56-39 0,-8 3 0,0 1 0,1 0 0,0 1 0,0 0 0,1 0 0,0 1 0,0 1 0,-11 14 0,4-3 0,-34 34 0,32-36 0,-33 41 0,14-8 0,-3-3 0,-81 78 0,109-114 0,2 1 0,0 0 0,0 1 0,1 0 0,1 1 0,1 0 0,0 0 0,1 1 0,1 0 0,-4 21 0,5-25 0,0 0 0,-1 0 0,0-1 0,-1 0 0,-16 22 0,-10 18 0,-3-4 0,29-40 0,0 1 0,0 0 0,-9 16 0,9-11-273,0-1 0,1 1 0,1 0 0,-5 21 0,6-12-6553</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="365.01">0 1004 24575,'0'-2'0,"1"1"0,0-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,4 1 0,48-6 0,-47 6 0,195 0 0,21-2 0,-195-1 0,1-1 0,-1-1 0,0-2 0,-1-1 0,0 0 0,0-2 0,-1-1 0,33-19 0,-44 23 0,0 1 0,0 1 0,0 0 0,1 1 0,0 0 0,0 1 0,19-1 0,-25 2 0,-3 1-124,-1 0 0,1-1 0,0 0 0,-1 0 0,0 0 0,1-1-1,-1 0 1,0 0 0,0 0 0,6-6 0,4-3-6702</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink106.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:25:10.409"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.3" units="cm"/>
+      <inkml:brushProperty name="height" value="0.6" units="cm"/>
+      <inkml:brushProperty name="color" value="#FFFC00"/>
+      <inkml:brushProperty name="tip" value="rectangle"/>
+      <inkml:brushProperty name="rasterOp" value="maskPen"/>
+      <inkml:brushProperty name="ignorePressure" value="1"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1,'8'0,"1"0,0 0,0 1,0 0,0 1,-1-1,1 2,-1-1,1 1,-1 1,0-1,0 1,0 1,-1 0,7 5,-3-3,-1 0,1-1,0 0,1-1,-1 0,1-1,0 0,0-1,0-1,13 2,33 8,25 2,32 3,-77-10,75 4,-102-12,1 1,0 1,-1 0,1 1,0 0,-1 1,0 0,0 1,0 0,11 6,-3-2,-1-2,1-1,0 0,0-1,0-1,0-1,36 0,54 8,22 4,-71-9,-49-3,-1 0,0 1,0 0,0 1,0 0,12 7,-11-5,0-1,0 0,1-1,18 5,74 0,-74-8,1 2,31 6,-24-2,1-2,-1-2,1-1,74-7,-108 4,0 0,-1 0,1-1,0 1,0-1,-1 0,1-1,-1 1,0-1,0 1,0-1,5-5,5-4</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink107.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:25:11.398"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.3" units="cm"/>
+      <inkml:brushProperty name="height" value="0.6" units="cm"/>
+      <inkml:brushProperty name="color" value="#FFFC00"/>
+      <inkml:brushProperty name="tip" value="rectangle"/>
+      <inkml:brushProperty name="rasterOp" value="maskPen"/>
+      <inkml:brushProperty name="ignorePressure" value="1"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1,'1807'0,"-1798"0,1 1,0 0,-1 1,1 0,-1 0,1 1,-1 0,0 1,0 0,-1 1,1-1,-1 2,11 7,-13-9,12 6,0-2,1-1,0 0,0-1,1-1,34 4,-11-1,-6-3,0-1,0-2,44-3,-46-1,1 2,-1 2,60 10,-58-5,1-1,73 2,-84-8</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink108.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:29.827"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
@@ -11766,7 +12515,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink101.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink109.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -11791,234 +12540,6 @@
     </inkml:brush>
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">49 141 24575,'0'-4'0,"1"-1"0,0 1 0,0 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,1 0 0,0 1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,7-2 0,9-4 0,1 1 0,0 0 0,34-5 0,54-8 0,-107 20 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,2 3 0,-2-2 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,-1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1 0 0,-1 7 0,-2 2 0,-1-1 0,0 1 0,-1-1 0,-1 1 0,0-1 0,0-1 0,-2 1 0,1-1 0,-16 18 0,-66 104 0,52-95 0,31-34 0,0 0 0,0 1 0,1 0 0,0 0 0,0 1 0,0-1 0,-4 10 0,3-6 0,0 0 0,-1 0 0,0 0 0,-12 12 0,11-14 0,0 0 0,1 1 0,1 1 0,-1-1 0,-8 20 0,9-18 0,0 0 0,0-1 0,-1 1 0,-1-1 0,-10 11 0,-16 22 0,34-42 0,-1-1 0,1 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,18 6 0,25-4 0,-40-3 0,44 1-109,1-2 1,0-1-1,-1-3 0,0-2 0,0-2 1,58-19-1,-70 18 109,0 2 0,1 1 0,0 2 0,40-1 0,27-3 0,2 1-15,-78 8 9,0-1 0,-1-2-1,1-1 1,0-1 0,32-10 0,-19 1-178,1 1 0,54-8 0,-72 18-6642</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink102.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:45.143"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">12 132 24575,'0'0'0,"-1"0"0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,-1-1 0,11-11 0,18-9 0,-15 14 0,2 1 0,-1 0 0,1 1 0,-1 1 0,1 0 0,31-3 0,-34 5 0,-1-1 0,1 0 0,-1-1 0,18-8 0,-19 7 0,1 1 0,-1 0 0,1 0 0,0 1 0,20-3 0,-18 5 0,0 0 0,1 0 0,-1 0 0,1 1 0,20 3 0,-31-2 0,0-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0 0 0,0-1 0,1 5 0,-1-1 0,0 1 0,0-1 0,0 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 0 0,-1 1 0,0-1 0,0-1 0,0 1 0,-1 0 0,0-1 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,-9 1 0,-11 4 0,0 1 0,-39 20 0,57-25 0,1 1 0,0-1 0,0 1 0,1 0 0,-1 1 0,1-1 0,0 1 0,1 1 0,-1-1 0,1 1 0,1-1 0,-7 14 0,-2-1 0,0 3 0,14-21 0,-1 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0-1 0,290-3 0,-283 2 0,1 0 0,0 0 0,-1-1 0,0 0 0,15-8 0,-15 7 0,0 0 0,0 1 0,0 0 0,1 0 0,-1 1 0,12-2 0,-18 4 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,1 1 0,-1-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,3 4 0,3 8 0,0-1 0,0 1 0,-2 1 0,1-1 0,2 19 0,-6-25 0,0 0 0,-1 0 0,0 1 0,0-1 0,-1 0 0,-1 1 0,1-1 0,-1 0 0,-1 0 0,1 1 0,-4 8 0,3-14 0,1 0 0,-1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-7 2 0,-46 18 0,47-20 0,-1 1 0,1 0 0,0 0 0,0 0 0,1 1 0,-1 1 0,-9 6 0,-2 8 0,14-14 0,0 1 0,0-1 0,-1-1 0,1 1 0,-1-1 0,0 0 0,-11 5 0,-58 29 0,44-21 0,-40 15 0,37-18-110,25-10 21,1 0-1,-2 0 0,1 0 1,0-1-1,-1 0 0,0-1 1,0 0-1,0-1 0,0 0 1,0 0-1,0-1 0,0 0 1,-11-2-1,5-3-6736</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink103.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:47.751"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">572 1 24575,'-17'0'0,"-6"-1"0,0 2 0,-42 6 0,58-5 0,-1-1 0,1 2 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 1 0,-10 10 0,-115 138 0,120-143 0,1 1 0,0-1 0,1 1 0,0 1 0,1 0 0,0 0 0,0 1 0,2 0 0,-8 19 0,10-25 0,1 1 0,-1-1 0,0 0 0,-1 0 0,0 0 0,0-1 0,-8 8 0,-19 27 0,29-37 0,0 0 0,0 0 0,0 0 0,-1 0 0,0-1 0,0 1 0,-5 2 0,-4 5 0,13-11 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,12 2 0,18-2 0,-30-1 0,31 1 0,57 9 0,-54-5 0,43 2 0,-75-7 0,16 0 0,-1 0 0,31-5 0,-43 4 0,1-1 0,-1 0 0,1 0 0,-1-1 0,0 1 0,0-1 0,0-1 0,-1 1 0,1-1 0,9-8 0,-5 4-119,0 1 0,1 0 1,0 0-1,1 1 0,14-5 0,-18 7-533,8-3-6174</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2773.83">307 97 24575,'25'-1'0,"-12"0"0,0 1 0,0 0 0,0 1 0,0 0 0,15 4 0,-26-4 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,-1 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,-1 4 0,-25 134 0,24-130 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-2 0 0,0-1 0,-8 13 0,-12 26 0,18-30 0,1 1 0,-6 27 0,8-26 0,-1-1 0,-12 30 0,13-39 0,0 0 0,0 1 0,1-1 0,1 1 0,0 0 0,0 0 0,1-1 0,1 17 0,0-23 0,0-1 0,0 1 0,0 0 0,1-1 0,0 1 0,-1-1 0,1 1 0,1-1 0,-1 1 0,0-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0-1 0,0 1 0,5 1 0,11 4-1365,-3 0-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink104.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:54.155"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">75 182 24575,'-3'239'0,"3"-236"0,0-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,4 0 0,13 4 0,0-1 0,0-1 0,23 1 0,-14-1 0,-24-3 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,-1 1 0,3 9 0,-3-8 0,0 1 0,-1 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,0 0 0,-1 0 0,1-1 0,-1 1 0,-1-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,-1 0 0,0-1 0,0 1 0,-7 7 0,-5 2 0,0-1 0,-21 15 0,24-20 0,0 1 0,0 1 0,0 0 0,-18 24 0,28-32 7,0 1 0,0-1-1,0 0 1,0 0 0,-1-1-1,1 1 1,-1-1 0,0 1-1,0-1 1,0 0 0,0-1 0,0 1-1,0-1 1,0 0 0,-5 1-1,-6 1-283,0-2 0,0 0 0,-15-2 0,22 1-87,-15-1-6462</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="838.32">101 108 24575,'108'1'0,"123"-3"0,-206-1-470,0-1 1,1-1-1,-2-2 0,38-14 0,-38 12 473,0 1-1,1 1 0,0 1 1,41-4-1,40-3 1224,-67 7-670,52-1-1,41 8-1920,-110-1-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink105.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:56.611"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1015 2 24575,'-93'-2'0,"-102"5"0,185-1 0,1 0 0,-1 1 0,0-1 0,0 2 0,1 0 0,-1 1 0,1 0 0,-9 6 0,6-3 0,-1-1 0,-1-1 0,-14 6 0,15-6 0,0-1 0,1 2 0,0 1 0,1-1 0,-1 1 0,1 1 0,0 0 0,1 1 0,0 0 0,-10 14 0,7-9 0,-1-1 0,-1 0 0,0-1 0,-21 14 0,22-19 0,1 0 0,1 1 0,0 0 0,-1 0 0,2 2 0,0-1 0,0 2 0,2-1 0,-1 2 0,1-2 0,0 3 0,1-2 0,1 2 0,0 0 0,1 0 0,1 0 0,-3 17 0,5-20 0,-1 1 0,0-1 0,0 1 0,-1-1 0,-1 0 0,0-1 0,0 1 0,-12 13 0,7-2 0,-1 1 0,2 0 0,1 0 0,0 1 0,-6 36 0,9-33 0,4-20 0,1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,0-2 0,1 1 0,0 1 0,0-2 0,0 1 0,1 0 0,-1-1 0,6 12 0,-5-14 0,0-1 0,0 1 0,1 0 0,-1 0 0,1 0 0,0-1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,1-2 0,-2 2 0,2-1 0,-1 1 0,1-1 0,5 0 0,37 2 0,2-2 0,65-7 0,-99 3 0,-1 1 0,-1-3 0,0 1 0,1-2 0,-1 0 0,0 1 0,20-16 0,-29 18 0,0-1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,2-12 0,9-65 0,-11 60 0,0 6 0,0-1 0,-2 1 0,0 0 0,0-1 0,-2 1 0,0 0 0,-5-19 0,5 31 0,0 0 0,0 2 0,-1-2 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 1 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 2 0,0-1 0,0 0 0,0 1 0,-1 0 0,1 0 0,-6-1 0,-11-1 0,0 1 0,-36 1 0,-257 2-1365,292-1-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink106.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:59.750"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 101 24575,'55'-19'0,"180"-14"0,-206 29 0,-1-1 0,30-10 0,-37 9 0,0 1 0,0 0 0,1 2 0,42-2 0,-62 5 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1 2 0,2 11 0,-1 0 0,-1 0 0,-3 32 0,1-22 0,1-3 0,1 8 0,-1 0 0,-2 0 0,-2-1 0,-16 58 0,20-81 0,0 0 0,0 0 0,0 1 0,1-1 0,0 0 0,1 1 0,-1-1 0,2 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,0 0 0,0-1 0,7 11 0,-3-3 0,0 0 0,8 28 0,-5 5-341,-2 1 0,-2 0-1,-2 89 1,-4-115-6485</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="482.01">242 595 24575,'17'-1'0,"0"-1"0,0 0 0,20-7 0,15-1 0,-34 6 0,0-1 0,0 0 0,-1-1 0,28-14 0,-23 10 0,46-15 0,-46 18 0,0-1 0,40-22 0,15-5 0,-67 31 0,12-5 0,1 0 0,-1 2 0,2 0 0,-1 2 0,1 1 0,39-3 0,-56 7-114,-1 0 1,1 0-1,-1-1 0,1 1 0,-1-2 1,0 1-1,1 0 0,-1-1 0,0 0 1,0-1-1,9-4 0,-3-2-6712</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink107.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:38:04.220"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">265 244 24575,'14'-2'0,"-13"2"0,-1 0 0,0 0 0,1-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,-1 1 0,1 0 0,-1 31 0,-1-2 0,1 0 0,1 1 0,2-1 0,1 0 0,2 0 0,0 0 0,12 35 0,-7-39 0,1 1 0,1-1 0,30 47 0,-34-59 0,-1 0 0,0 0 0,-1 0 0,6 22 0,4 9 0,-14-40 0,0 0 0,0 0 0,0 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,-1 1 0,-1 5 0,-2-3 0,1 0 0,-1 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,0-1 0,-8 8 0,6-8 0,1 0 0,-1 0 0,0-1 0,0 1 0,-1-2 0,-13 8 0,-9 4 0,20-10 0,0 1 0,-1-1 0,0 0 0,0-1 0,-11 4 0,16-7 0,1-1 0,-1 0 0,0-1 0,1 1 0,-1-1 0,0 0 0,1-1 0,-1 1 0,1-1 0,-1 0 0,-8-3 0,5 2 0,0-1 0,0 0 0,0-1 0,0 0 0,0 0 0,1-1 0,0 0 0,-13-10 0,-2-2 0,17 14 0,0-1 0,0-1 0,0 1 0,1-1 0,0 0 0,0 0 0,-6-8 0,10 11 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,4-3 0,15-18 0,1 2 0,0 0 0,48-34 0,-10 8 0,-19 20 0,-33 23 0,0-1 0,0 0 0,0 1 0,-1-2 0,0 1 0,0-1 0,0 0 0,8-11 0,-11 11 0,1 0 0,0 1 0,1 0 0,-1 0 0,1 1 0,0-1 0,0 1 0,0 0 0,1 0 0,0 0 0,-1 1 0,1 0 0,9-3 0,16-10 0,-23 11 0,0 0 0,-1-1 0,1 0 0,-1-1 0,-1 0 0,1 0 0,9-15 0,-10 14 0,0 0 0,0 1 0,1-1 0,0 1 0,0 1 0,1-1 0,11-7 0,89-58 0,-60 38 0,-33 26 0,1 0 0,1 2 0,-1 0 0,1 1 0,0 1 0,0 0 0,1 1 0,-1 1 0,23 0 0,-27 2 0,-1-1 0,1 0 0,-1-1 0,1 0 0,-1-1 0,19-7 0,-28 9 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,-1-2 0,1 1 0,-1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,-1 0 0,0-5 0,-1 1 0,0 0 0,0-1 0,-1 1 0,0 0 0,0 1 0,-1-1 0,0 0 0,0 1 0,0 0 0,-1 0 0,0 0 0,-8-7 0,-7-5 0,0 1 0,-28-19 0,37 31 0,-1-1 0,1 2 0,-1-1 0,0 2 0,0 0 0,0 0 0,-20-1 0,-6-3 0,-4 1 0,-1 2 0,1 2 0,-58 4 0,19 0 0,49 0 0,-55 9 0,55-5 0,-55 2 0,34-8-1365,31 0-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink108.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:38:08.194"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1430 57 24575,'-169'-13'0,"-6"0"0,130 13 0,0-1 0,-75-13 0,69 7 0,0 2 0,0 2 0,0 3 0,-61 6 0,102-5 0,0 0 0,0 1 0,0 1 0,0-1 0,1 1 0,-1 1 0,1 0 0,0 0 0,0 1 0,0 0 0,0 1 0,1-1 0,0 2 0,0-1 0,1 1 0,0 0 0,-10 12 0,-19 19 0,29-31 0,-1 0 0,1 0 0,1 1 0,0 0 0,-10 14 0,-3 15 0,1 0 0,-18 57 0,31-80 0,1 0 0,1 0 0,1 0 0,0 1 0,1-1 0,0 0 0,1 1 0,1-1 0,0 1 0,6 21 0,-5-31 0,0 0 0,1 0 0,0 0 0,0-1 0,0 0 0,0 1 0,1-1 0,0 0 0,0 0 0,0-1 0,0 1 0,0-1 0,1 0 0,0 0 0,0 0 0,-1-1 0,2 0 0,-1 0 0,8 3 0,11 2 0,0 0 0,48 6 0,1-7 0,141-6 0,-87-3 0,-95 3 0,-1-2 0,0-1 0,0-2 0,45-12 0,-56 12 0,-1-2 0,0 0 0,-1-1 0,1-1 0,-1-1 0,-1-1 0,31-23 0,29-23 0,-59 46 0,0-2 0,-1 0 0,-1 0 0,0-2 0,15-17 0,-3 3 0,-24 26 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,2-6 0,-2 4 0,3-8 0,-2 1 0,0 0 0,0-1 0,0-27 0,-3 39 0,0 1 0,0 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,-2-3 0,2 4 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,-3 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,0 1 0,0-1 0,-1 1 0,2 0 0,-1 0 0,0 0 0,1 1 0,-1 0 0,1-1 0,0 2 0,0-1 0,1 0 0,-1 1 0,1-1 0,0 1 0,0 0 0,-2 7 0,-2 7 0,2-1 0,0 1 0,1 0 0,-1 31 0,-3 8 0,-1-3 0,3-14 0,-2 0 0,-16 48 0,-6-35 0,25-47 0,0 1 0,1-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-3 13 0,3 6 0,2-1 0,0 0 0,5 38 0,-2-41 0,0-1 0,-2 1 0,-1 0 0,0 0 0,-6 23 0,3-35 0,-1-1 0,0 0 0,0 0 0,-1-1 0,-1 1 0,0-1 0,-15 16 0,-2 4 0,-3-3 0,22-23 0,2 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,1 0 0,0 0 0,-4 8 0,-74 135 0,68-132 0,1 0 0,-2-1 0,0 0 0,0-1 0,-2-1 0,1 0 0,-34 18 0,26-20 0,0 0 0,-1-2 0,-1 0 0,1-2 0,-1-1 0,-1 0 0,-40 1 0,-31 6 0,74-8 0,0-1 0,-1-1 0,1-1 0,-1-1 0,1-1 0,-1-1 0,1-2 0,0 0 0,0-1 0,-36-13 0,46 15 21,0 0-1,0 0 0,-24 0 1,27 2-202,0 1 0,0-2 0,1 1 0,-1-1 0,0-1 1,1 0-1,-17-7 0,9 0-6645</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink109.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:38:11.360"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">280 1 24575,'1'67'0,"-3"77"0,0-134 0,0 1 0,-1-1 0,0 0 0,0 0 0,-10 18 0,8-18 0,1 0 0,0 1 0,0-1 0,1 1 0,-3 19 0,4-16 0,-1 0 0,-1 0 0,0 0 0,-12 26 0,-7 21 0,15-35 0,-23 48 0,1-5 0,20-34 0,9-29 0,0-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1-1 0,-4 6 0,3-5-14,1 0 1,-1 1-1,1-1 0,0 1 0,0 0 1,1 1-1,-1-1 0,1 0 0,1 1 1,0 0-1,-4 13 0,-2 9-1186,2-13-5626</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="764.22">751 344 24575,'-11'1'0,"1"-1"0,-1 1 0,1 1 0,-1 0 0,1 0 0,0 1 0,0 0 0,0 1 0,0 0 0,1 1 0,0 0 0,-1 0 0,2 1 0,-1 0 0,-14 14 0,0 3 0,18-19 0,0 0 0,0 1 0,1 0 0,0-1 0,0 2 0,0-1 0,-4 9 0,3-6 0,0 1 0,-1-2 0,1 1 0,-2 0 0,1-1 0,-12 9 0,13-11 0,0-1 0,0 1 0,0 0 0,0 0 0,1 1 0,0-1 0,0 1 0,0 0 0,1 0 0,0 1 0,0-1 0,0 1 0,-2 11 0,2-6 0,1 0 0,-2-1 0,0 1 0,0-1 0,-1 0 0,0 0 0,-1 0 0,0-1 0,-12 15 0,10-12 0,1-1 0,1 1 0,0 0 0,0 1 0,2-1 0,-1 1 0,2 0 0,0 0 0,1 0 0,0 0 0,1 1 0,0-1 0,1 1 0,4 21 0,-4-34 0,1 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,6 1 0,8 0 0,1 0 0,-1 0 0,19-3 0,-16 1 0,194-2 0,-199 0 0,1 0 0,0-1 0,-1-1 0,0-1 0,-1 0 0,1 0 0,12-9 0,36-16 0,-26 14 0,0-1 0,44-33 0,4-1 0,-77 48 0,-1-1 0,0 1 0,-1-1 0,1-1 0,-1 1 0,0-1 0,0 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,-1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,0-1 0,1-14 0,1-12 0,-2-1 0,-5-67 0,1 38 0,2 41 0,1 14 0,-1 0 0,0 0 0,-1-1 0,0 1 0,-3-13 0,4 19 0,-1 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,-3-1 0,-62-10 0,0 3 0,-92 1 0,133 7-1365,3 1-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -12066,6 +12587,234 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:45.143"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">12 132 24575,'0'0'0,"-1"0"0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,-1-1 0,11-11 0,18-9 0,-15 14 0,2 1 0,-1 0 0,1 1 0,-1 1 0,1 0 0,31-3 0,-34 5 0,-1-1 0,1 0 0,-1-1 0,18-8 0,-19 7 0,1 1 0,-1 0 0,1 0 0,0 1 0,20-3 0,-18 5 0,0 0 0,1 0 0,-1 0 0,1 1 0,20 3 0,-31-2 0,0-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0 0 0,0-1 0,1 5 0,-1-1 0,0 1 0,0-1 0,0 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 0 0,-1 1 0,0-1 0,0-1 0,0 1 0,-1 0 0,0-1 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 1 0,-9 1 0,-11 4 0,0 1 0,-39 20 0,57-25 0,1 1 0,0-1 0,0 1 0,1 0 0,-1 1 0,1-1 0,0 1 0,1 1 0,-1-1 0,1 1 0,1-1 0,-7 14 0,-2-1 0,0 3 0,14-21 0,-1 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0-1 0,290-3 0,-283 2 0,1 0 0,0 0 0,-1-1 0,0 0 0,15-8 0,-15 7 0,0 0 0,0 1 0,0 0 0,1 0 0,-1 1 0,12-2 0,-18 4 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,1 1 0,-1-1 0,-1 1 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,3 4 0,3 8 0,0-1 0,0 1 0,-2 1 0,1-1 0,2 19 0,-6-25 0,0 0 0,-1 0 0,0 1 0,0-1 0,-1 0 0,-1 1 0,1-1 0,-1 0 0,-1 0 0,1 1 0,-4 8 0,3-14 0,1 0 0,-1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-7 2 0,-46 18 0,47-20 0,-1 1 0,1 0 0,0 0 0,0 0 0,1 1 0,-1 1 0,-9 6 0,-2 8 0,14-14 0,0 1 0,0-1 0,-1-1 0,1 1 0,-1-1 0,0 0 0,-11 5 0,-58 29 0,44-21 0,-40 15 0,37-18-110,25-10 21,1 0-1,-2 0 0,1 0 1,0-1-1,-1 0 0,0-1 1,0 0-1,0-1 0,0 0 1,0 0-1,0-1 0,0 0 1,-11-2-1,5-3-6736</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink111.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:47.751"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">572 1 24575,'-17'0'0,"-6"-1"0,0 2 0,-42 6 0,58-5 0,-1-1 0,1 2 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 1 0,-10 10 0,-115 138 0,120-143 0,1 1 0,0-1 0,1 1 0,0 1 0,1 0 0,0 0 0,0 1 0,2 0 0,-8 19 0,10-25 0,1 1 0,-1-1 0,0 0 0,-1 0 0,0 0 0,0-1 0,-8 8 0,-19 27 0,29-37 0,0 0 0,0 0 0,0 0 0,-1 0 0,0-1 0,0 1 0,-5 2 0,-4 5 0,13-11 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,12 2 0,18-2 0,-30-1 0,31 1 0,57 9 0,-54-5 0,43 2 0,-75-7 0,16 0 0,-1 0 0,31-5 0,-43 4 0,1-1 0,-1 0 0,1 0 0,-1-1 0,0 1 0,0-1 0,0-1 0,-1 1 0,1-1 0,9-8 0,-5 4-119,0 1 0,1 0 1,0 0-1,1 1 0,14-5 0,-18 7-533,8-3-6174</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2773.83">307 97 24575,'25'-1'0,"-12"0"0,0 1 0,0 0 0,0 1 0,0 0 0,15 4 0,-26-4 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,-1 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,-1 4 0,-25 134 0,24-130 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-2 0 0,0-1 0,-8 13 0,-12 26 0,18-30 0,1 1 0,-6 27 0,8-26 0,-1-1 0,-12 30 0,13-39 0,0 0 0,0 1 0,1-1 0,1 1 0,0 0 0,0 0 0,1-1 0,1 17 0,0-23 0,0-1 0,0 1 0,0 0 0,1-1 0,0 1 0,-1-1 0,1 1 0,1-1 0,-1 1 0,0-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0-1 0,0 1 0,5 1 0,11 4-1365,-3 0-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink112.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:54.155"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">75 182 24575,'-3'239'0,"3"-236"0,0-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,4 0 0,13 4 0,0-1 0,0-1 0,23 1 0,-14-1 0,-24-3 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,-1 1 0,3 9 0,-3-8 0,0 1 0,-1 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,0 0 0,-1 0 0,1-1 0,-1 1 0,-1-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,-1 0 0,0-1 0,0 1 0,-7 7 0,-5 2 0,0-1 0,-21 15 0,24-20 0,0 1 0,0 1 0,0 0 0,-18 24 0,28-32 7,0 1 0,0-1-1,0 0 1,0 0 0,-1-1-1,1 1 1,-1-1 0,0 1-1,0-1 1,0 0 0,0-1 0,0 1-1,0-1 1,0 0 0,-5 1-1,-6 1-283,0-2 0,0 0 0,-15-2 0,22 1-87,-15-1-6462</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="838.32">101 108 24575,'108'1'0,"123"-3"0,-206-1-470,0-1 1,1-1-1,-2-2 0,38-14 0,-38 12 473,0 1-1,1 1 0,0 1 1,41-4-1,40-3 1224,-67 7-670,52-1-1,41 8-1920,-110-1-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink113.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:56.611"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1015 2 24575,'-93'-2'0,"-102"5"0,185-1 0,1 0 0,-1 1 0,0-1 0,0 2 0,1 0 0,-1 1 0,1 0 0,-9 6 0,6-3 0,-1-1 0,-1-1 0,-14 6 0,15-6 0,0-1 0,1 2 0,0 1 0,1-1 0,-1 1 0,1 1 0,0 0 0,1 1 0,0 0 0,-10 14 0,7-9 0,-1-1 0,-1 0 0,0-1 0,-21 14 0,22-19 0,1 0 0,1 1 0,0 0 0,-1 0 0,2 2 0,0-1 0,0 2 0,2-1 0,-1 2 0,1-2 0,0 3 0,1-2 0,1 2 0,0 0 0,1 0 0,1 0 0,-3 17 0,5-20 0,-1 1 0,0-1 0,0 1 0,-1-1 0,-1 0 0,0-1 0,0 1 0,-12 13 0,7-2 0,-1 1 0,2 0 0,1 0 0,0 1 0,-6 36 0,9-33 0,4-20 0,1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,0-2 0,1 1 0,0 1 0,0-2 0,0 1 0,1 0 0,-1-1 0,6 12 0,-5-14 0,0-1 0,0 1 0,1 0 0,-1 0 0,1 0 0,0-1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,1-2 0,-2 2 0,2-1 0,-1 1 0,1-1 0,5 0 0,37 2 0,2-2 0,65-7 0,-99 3 0,-1 1 0,-1-3 0,0 1 0,1-2 0,-1 0 0,0 1 0,20-16 0,-29 18 0,0-1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,2-12 0,9-65 0,-11 60 0,0 6 0,0-1 0,-2 1 0,0 0 0,0-1 0,-2 1 0,0 0 0,-5-19 0,5 31 0,0 0 0,0 2 0,-1-2 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 1 0,1 0 0,-1 0 0,0 0 0,0-1 0,0 2 0,0-1 0,0 0 0,0 1 0,-1 0 0,1 0 0,-6-1 0,-11-1 0,0 1 0,-36 1 0,-257 2-1365,292-1-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink114.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:37:59.750"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 101 24575,'55'-19'0,"180"-14"0,-206 29 0,-1-1 0,30-10 0,-37 9 0,0 1 0,0 0 0,1 2 0,42-2 0,-62 5 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1 2 0,2 11 0,-1 0 0,-1 0 0,-3 32 0,1-22 0,1-3 0,1 8 0,-1 0 0,-2 0 0,-2-1 0,-16 58 0,20-81 0,0 0 0,0 0 0,0 1 0,1-1 0,0 0 0,1 1 0,-1-1 0,2 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,0 0 0,0-1 0,7 11 0,-3-3 0,0 0 0,8 28 0,-5 5-341,-2 1 0,-2 0-1,-2 89 1,-4-115-6485</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="482.01">242 595 24575,'17'-1'0,"0"-1"0,0 0 0,20-7 0,15-1 0,-34 6 0,0-1 0,0 0 0,-1-1 0,28-14 0,-23 10 0,46-15 0,-46 18 0,0-1 0,40-22 0,15-5 0,-67 31 0,12-5 0,1 0 0,-1 2 0,2 0 0,-1 2 0,1 1 0,39-3 0,-56 7-114,-1 0 1,1 0-1,-1-1 0,1 1 0,-1-2 1,0 1-1,1 0 0,-1-1 0,0 0 1,0-1-1,9-4 0,-3-2-6712</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink115.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:38:04.220"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">265 244 24575,'14'-2'0,"-13"2"0,-1 0 0,0 0 0,1-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,-1 1 0,1 0 0,-1 31 0,-1-2 0,1 0 0,1 1 0,2-1 0,1 0 0,2 0 0,0 0 0,12 35 0,-7-39 0,1 1 0,1-1 0,30 47 0,-34-59 0,-1 0 0,0 0 0,-1 0 0,6 22 0,4 9 0,-14-40 0,0 0 0,0 0 0,0 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,-1 1 0,-1 5 0,-2-3 0,1 0 0,-1 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,0-1 0,-8 8 0,6-8 0,1 0 0,-1 0 0,0-1 0,0 1 0,-1-2 0,-13 8 0,-9 4 0,20-10 0,0 1 0,-1-1 0,0 0 0,0-1 0,-11 4 0,16-7 0,1-1 0,-1 0 0,0-1 0,1 1 0,-1-1 0,0 0 0,1-1 0,-1 1 0,1-1 0,-1 0 0,-8-3 0,5 2 0,0-1 0,0 0 0,0-1 0,0 0 0,0 0 0,1-1 0,0 0 0,-13-10 0,-2-2 0,17 14 0,0-1 0,0-1 0,0 1 0,1-1 0,0 0 0,0 0 0,-6-8 0,10 11 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,0-1 0,-1 1 0,1 0 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,4-3 0,15-18 0,1 2 0,0 0 0,48-34 0,-10 8 0,-19 20 0,-33 23 0,0-1 0,0 0 0,0 1 0,-1-2 0,0 1 0,0-1 0,0 0 0,8-11 0,-11 11 0,1 0 0,0 1 0,1 0 0,-1 0 0,1 1 0,0-1 0,0 1 0,0 0 0,1 0 0,0 0 0,-1 1 0,1 0 0,9-3 0,16-10 0,-23 11 0,0 0 0,-1-1 0,1 0 0,-1-1 0,-1 0 0,1 0 0,9-15 0,-10 14 0,0 0 0,0 1 0,1-1 0,0 1 0,0 1 0,1-1 0,11-7 0,89-58 0,-60 38 0,-33 26 0,1 0 0,1 2 0,-1 0 0,1 1 0,0 1 0,0 0 0,1 1 0,-1 1 0,23 0 0,-27 2 0,-1-1 0,1 0 0,-1-1 0,1 0 0,-1-1 0,19-7 0,-28 9 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,-1-2 0,1 1 0,-1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,-1 0 0,0-5 0,-1 1 0,0 0 0,0-1 0,-1 1 0,0 0 0,0 1 0,-1-1 0,0 0 0,0 1 0,0 0 0,-1 0 0,0 0 0,-8-7 0,-7-5 0,0 1 0,-28-19 0,37 31 0,-1-1 0,1 2 0,-1-1 0,0 2 0,0 0 0,0 0 0,-20-1 0,-6-3 0,-4 1 0,-1 2 0,1 2 0,-58 4 0,19 0 0,49 0 0,-55 9 0,55-5 0,-55 2 0,34-8-1365,31 0-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink116.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:38:08.194"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1430 57 24575,'-169'-13'0,"-6"0"0,130 13 0,0-1 0,-75-13 0,69 7 0,0 2 0,0 2 0,0 3 0,-61 6 0,102-5 0,0 0 0,0 1 0,0 1 0,0-1 0,1 1 0,-1 1 0,1 0 0,0 0 0,0 1 0,0 0 0,0 1 0,1-1 0,0 2 0,0-1 0,1 1 0,0 0 0,-10 12 0,-19 19 0,29-31 0,-1 0 0,1 0 0,1 1 0,0 0 0,-10 14 0,-3 15 0,1 0 0,-18 57 0,31-80 0,1 0 0,1 0 0,1 0 0,0 1 0,1-1 0,0 0 0,1 1 0,1-1 0,0 1 0,6 21 0,-5-31 0,0 0 0,1 0 0,0 0 0,0-1 0,0 0 0,0 1 0,1-1 0,0 0 0,0 0 0,0-1 0,0 1 0,0-1 0,1 0 0,0 0 0,0 0 0,-1-1 0,2 0 0,-1 0 0,8 3 0,11 2 0,0 0 0,48 6 0,1-7 0,141-6 0,-87-3 0,-95 3 0,-1-2 0,0-1 0,0-2 0,45-12 0,-56 12 0,-1-2 0,0 0 0,-1-1 0,1-1 0,-1-1 0,-1-1 0,31-23 0,29-23 0,-59 46 0,0-2 0,-1 0 0,-1 0 0,0-2 0,15-17 0,-3 3 0,-24 26 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,2-6 0,-2 4 0,3-8 0,-2 1 0,0 0 0,0-1 0,0-27 0,-3 39 0,0 1 0,0 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,-2-3 0,2 4 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,-1 1 0,-3 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,0 1 0,0-1 0,-1 1 0,2 0 0,-1 0 0,0 0 0,1 1 0,-1 0 0,1-1 0,0 2 0,0-1 0,1 0 0,-1 1 0,1-1 0,0 1 0,0 0 0,-2 7 0,-2 7 0,2-1 0,0 1 0,1 0 0,-1 31 0,-3 8 0,-1-3 0,3-14 0,-2 0 0,-16 48 0,-6-35 0,25-47 0,0 1 0,1-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-3 13 0,3 6 0,2-1 0,0 0 0,5 38 0,-2-41 0,0-1 0,-2 1 0,-1 0 0,0 0 0,-6 23 0,3-35 0,-1-1 0,0 0 0,0 0 0,-1-1 0,-1 1 0,0-1 0,-15 16 0,-2 4 0,-3-3 0,22-23 0,2 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,1 0 0,0 0 0,-4 8 0,-74 135 0,68-132 0,1 0 0,-2-1 0,0 0 0,0-1 0,-2-1 0,1 0 0,-34 18 0,26-20 0,0 0 0,-1-2 0,-1 0 0,1-2 0,-1-1 0,-1 0 0,-40 1 0,-31 6 0,74-8 0,0-1 0,-1-1 0,1-1 0,-1-1 0,1-1 0,-1-1 0,1-2 0,0 0 0,0-1 0,-36-13 0,46 15 21,0 0-1,0 0 0,-24 0 1,27 2-202,0 1 0,0-2 0,1 1 0,-1-1 0,0-1 1,1 0-1,-17-7 0,9 0-6645</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink117.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:38:11.360"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">280 1 24575,'1'67'0,"-3"77"0,0-134 0,0 1 0,-1-1 0,0 0 0,0 0 0,-10 18 0,8-18 0,1 0 0,0 1 0,0-1 0,1 1 0,-3 19 0,4-16 0,-1 0 0,-1 0 0,0 0 0,-12 26 0,-7 21 0,15-35 0,-23 48 0,1-5 0,20-34 0,9-29 0,0-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1-1 0,-4 6 0,3-5-14,1 0 1,-1 1-1,1-1 0,0 1 0,0 0 1,1 1-1,-1-1 0,1 0 0,1 1 1,0 0-1,-4 13 0,-2 9-1186,2-13-5626</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="764.22">751 344 24575,'-11'1'0,"1"-1"0,-1 1 0,1 1 0,-1 0 0,1 0 0,0 1 0,0 0 0,0 1 0,0 0 0,1 1 0,0 0 0,-1 0 0,2 1 0,-1 0 0,-14 14 0,0 3 0,18-19 0,0 0 0,0 1 0,1 0 0,0-1 0,0 2 0,0-1 0,-4 9 0,3-6 0,0 1 0,-1-2 0,1 1 0,-2 0 0,1-1 0,-12 9 0,13-11 0,0-1 0,0 1 0,0 0 0,0 0 0,1 1 0,0-1 0,0 1 0,0 0 0,1 0 0,0 1 0,0-1 0,0 1 0,-2 11 0,2-6 0,1 0 0,-2-1 0,0 1 0,0-1 0,-1 0 0,0 0 0,-1 0 0,0-1 0,-12 15 0,10-12 0,1-1 0,1 1 0,0 0 0,0 1 0,2-1 0,-1 1 0,2 0 0,0 0 0,1 0 0,0 0 0,1 1 0,0-1 0,1 1 0,4 21 0,-4-34 0,1 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,6 1 0,8 0 0,1 0 0,-1 0 0,19-3 0,-16 1 0,194-2 0,-199 0 0,1 0 0,0-1 0,-1-1 0,0-1 0,-1 0 0,1 0 0,12-9 0,36-16 0,-26 14 0,0-1 0,44-33 0,4-1 0,-77 48 0,-1-1 0,0 1 0,-1-1 0,1-1 0,-1 1 0,0-1 0,0 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,-1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,0-1 0,1-14 0,1-12 0,-2-1 0,-5-67 0,1 38 0,2 41 0,1 14 0,-1 0 0,0 0 0,-1-1 0,0 1 0,-3-13 0,4 19 0,-1 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,-3-1 0,-62-10 0,0 3 0,-92 1 0,133 7-1365,3 1-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink118.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:38:14.376"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
@@ -12078,7 +12827,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink111.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink119.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -12107,7 +12856,35 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink112.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink12.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T04:27:13.561"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">224 0 24575,'-7'1'0,"1"0"0,-1 1 0,1-1 0,0 1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,1 1 0,-1-1 0,1 1 0,-7 7 0,-18 11 0,23-18 0,0 1 0,1 1 0,0-1 0,0 1 0,0 0 0,1 0 0,0 1 0,0 0 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,-3 15 0,1 5 0,0 1 0,-2 54 0,6-50 0,1-18 0,0-13 0,1 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 4 0,1-5 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,5 0 0,17 5 0,0-2 0,1 0 0,-1-2 0,1 0 0,0-2 0,0-1 0,47-7 0,-70 7 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0-1 0,-1 1 0,3-4 0,18-19 0,3 10 0,-23 15 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,2-3 0,3-18 0,7-33 0,7-84 0,-18 76 0,1 140 0,-15 145 0,11-207 0,2 1 0,0 0 0,1 0 0,4 27 0,2 28 0,-6-6 0,-3 91 0,2-153 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,-4 1 0,-9 1 0,-1-1 0,0-1 0,1 0 0,-20-3 0,-5 0 0,-105 3-1365,131 0-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink120.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -12133,34 +12910,6 @@
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">0 138 24575,'0'452'0,"1"-441"0,0 0 0,1-1 0,1 0 0,-1 1 0,1-1 0,1 0 0,6 14 0,-4-13 0,-2 1 0,1-1 0,-2 1 0,1 1 0,1 15 0,-3 167 71,-4-99-1507,2-74-5390</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="738">413 185 24575,'0'-2'0,"1"-1"0,-1 0 0,1 1 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,4-1 0,44-25 0,-37 22 0,-1-1 0,0 0 0,0-1 0,-1 0 0,16-15 0,13-9 0,-38 30 0,0 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,-1 0 0,4 3 0,-2 0 0,1 0 0,-1 1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,-1 0 0,0-1 0,0 1 0,3 11 0,7 44 0,-1 0 0,1 68 0,-9-98 0,9 42 0,-8-53 0,0 1 0,1 25 0,-5-46 0,1 29 0,-5 55 0,2-73 0,0 0 0,-1 0 0,0-1 0,0 0 0,-1 1 0,-1-1 0,0 0 0,-7 11 0,7-12 0,-1 0 0,0-1 0,0 1 0,-1-1 0,0-1 0,0 1 0,-1-1 0,0-1 0,0 1 0,-1-1 0,0-1 0,0 0 0,-11 5 0,13-6 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 1 0,0 0 0,1 1 0,-1-1 0,1 1 0,1 0 0,-1 0 0,1 1 0,0-1 0,-4 10 0,8-15 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,37 3 0,-35-2 0,30 0 0,161-4 0,-184 2 0,0 0 0,-1-1 0,1 0 0,-1-1 0,15-6 0,-14 4 0,1 2 0,-1-1 0,1 2 0,14-3 0,52-1 0,-59 6 0,1 0 0,-1-1 0,0-1 0,0-1 0,27-9 0,12-9-455,1 2 0,67-13 0,-107 30-6371</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink12.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T04:27:13.561"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">224 0 24575,'-7'1'0,"1"0"0,-1 1 0,1-1 0,0 1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,1 1 0,-1-1 0,1 1 0,-7 7 0,-18 11 0,23-18 0,0 1 0,1 1 0,0-1 0,0 1 0,0 0 0,1 0 0,0 1 0,0 0 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,-3 15 0,1 5 0,0 1 0,-2 54 0,6-50 0,1-18 0,0-13 0,1 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 4 0,1-5 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,5 0 0,17 5 0,0-2 0,1 0 0,-1-2 0,1 0 0,0-2 0,0-1 0,47-7 0,-70 7 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0-1 0,-1 1 0,3-4 0,18-19 0,3 10 0,-23 15 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,2-3 0,3-18 0,7-33 0,7-84 0,-18 76 0,1 140 0,-15 145 0,11-207 0,2 1 0,0 0 0,1 0 0,4 27 0,2 28 0,-6-6 0,-3 91 0,2-153 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,-4 1 0,-9 1 0,-1-1 0,0-1 0,1 0 0,-20-3 0,-5 0 0,-105 3-1365,131 0-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -13867,15 +14616,15 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:24.076"/>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-20T02:31:58.324"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
       <inkml:brushProperty name="width" value="0.035" units="cm"/>
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 740 24575,'1'-8'5,"-1"1"1,1-1-1,0 0 0,0 1 0,1 0 0,-1-1 1,2 1-1,-1 0 0,1 0 0,0 0 0,0 0 1,1 1-1,-1-1 0,9-9 0,2 0-174,1 0 0,1 0 0,25-18 0,-25 22 95,0-1-1,-1-1 1,0-1-1,14-18 1,-14 10 74,-5 9 0,0 0 0,1 0 0,0 1 0,21-19 0,-22 22-6,1-1 0,-1 0 0,-1 0 0,0-1 0,-1-1 0,0 0 0,7-14 0,27-41 862,-37 62-830,0 0-1,1 1 0,0-1 0,0 2 1,0-1-1,13-6 0,-13 7-27,0 0 0,1 0 0,-1 0 1,-1-1-1,1 0 0,-1 0 0,9-11 0,1-12 2,-13 24 0,-1 0 0,1 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,0 1 0,0 0 0,0 0 0,5-3 0,-8 6 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,0 1 0,0 1 0,6 35 0,-6-35 0,3 385 0,-7-192 0,5 115-1365,-1-265-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 160 24575,'0'-2'0,"1"0"0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,2-1 0,15-13 0,14-16 0,-29 29 0,-1-1 0,1 1 0,-1-1 0,0 0 0,0 1 0,0-2 0,-1 1 0,1 0 0,-1 0 0,0-1 0,1 1 0,-1-1 0,-1 0 0,1 1 0,-1-1 0,2-6 0,-3 9 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,1-1 0,-1 2 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 1 0,3 42 0,-3 65 0,-2-39 0,2-67-91,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,-5 2 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="841.26">23 533 24575,'6'-5'0,"0"0"0,0 1 0,1-1 0,-1 1 0,1 0 0,0 1 0,0 0 0,0 0 0,0 0 0,14-2 0,-15 4 0,0 0 0,0 0 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 1 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1 0 0,-1 0 0,10 5 0,-14-6 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,-5 6 0,0-1 0,-1 1 0,-11 10 0,8-7 0,-5 6 0,12-13 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0-1 0,0 1 0,-1 0 0,1-1 0,0 0 0,-9 3 0,11-4 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,1-1 0,-1 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 2 0,1-4 0,1 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0-1 0,12 3 0,-1 0 0,1 1 0,14 5 0,-16-4 0,1-1 0,-1 0 0,1-1 0,16 1 0,18-3-1365,-40 0-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -13895,15 +14644,23 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:26.173"/>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-20T02:32:00.124"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
       <inkml:brushProperty name="width" value="0.035" units="cm"/>
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 1 24575,'0'0'-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">185 72 24575,'0'-2'0,"0"0"0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,4-1 0,5-1 0,0 1 0,0 0 0,0 0 0,15 1 0,-17 1 0,0-1 0,1 0 0,-1 0 0,12-4 0,-10 2 0,1 1 0,-1 1 0,0 0 0,0 0 0,1 1 0,-1 0 0,15 3 0,-25-2 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,0-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-2 1 0,-16 42 0,18-42 0,-2 1 0,-1 4 0,-1-1 0,1 0 0,-1 0 0,-9 11 0,11-15 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0-1 0,-6 1 0,-18 7 0,23-7 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-8-1 0,48 0 0,-24-1 0,1 0 0,-1 1 0,0 1 0,0 0 0,1 1 0,19 5 0,-30-5 0,-1-1 0,1 0 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 5 0,0-2 0,0 0 0,-1 1 0,1-1 0,-1 0 0,0 0 0,0 1 0,0-1 0,-3 5 0,0-6 0,0 0 0,0-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1-1 0,-1 0 0,-1 0 0,1 0 0,0-1 0,-9 2 0,-10 4 0,-3 3 0,0-2 0,-44 7 0,45-13 15,-1-1 0,-31-2 0,8 0-1425,41 1-5416</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="871.95">931 369 24575,'-8'6'0,"0"1"0,0-1 0,-18 10 0,-19 14 0,38-24 0,0 0 0,-1-1 0,0 0 0,-13 6 0,14-8 0,0 0 0,1 1 0,-1 0 0,1 0 0,0 0 0,0 1 0,0 0 0,-6 7 0,4-2 0,0 0 0,-1-1 0,0 0 0,-1-1 0,0 0 0,0 0 0,0-1 0,-13 6 0,22-13 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,1 0 0,-2 1 0,19 6 0,-7-5 0,4 1 0,0 0 0,27 3 0,22 5 0,-42-8 0,0 0 0,0-1 0,0-2 0,0 0 0,41-4 0,-1 1 0,-34 4 0,-19-1 0,-1-1 0,1 1 0,0-1 0,-1-1 0,1 1 0,15-4 0,-22 3-25,0 0-1,0 0 0,0 0 0,-1 0 1,1 0-1,0 0 0,0 0 1,-1-1-1,1 1 0,-1 0 1,1 0-1,-1 0 0,1-1 0,-1 1 1,0 0-1,0-1 0,0 1 1,1 0-1,-1-1 0,0 1 1,-1 0-1,1-1 0,0 1 0,-1-2 1,1-1-698,0-3-6103</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1239.67">984 429 24575,'-22'39'0,"12"16"0,-4 27 0,3-38 0,9-38 0,0 1 0,0-1 0,0 1 0,1-1 0,0 1 0,0 9 0,1-10 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,-1 0 0,1-1 0,-5 12 0,3-17-1365</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2266.52">56 1061 24575,'1'1'0,"0"-1"0,1 0 0,-1 1 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0 1 0,1-1 0,-1 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,-2 4 0,-1-5 0,14-1 0,1 5 0,-1 1 0,0 0 0,0 0 0,13 9 0,-17-10 0,-4-3 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 3 0,5 23 0,-3-20 0,1 0 0,-1 0 0,0 0 0,-1 1 0,1 15 0,-2-22 0,0-1 0,-1 1 0,1-1 0,0 1 0,-1 0 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,-2 0 0,-12-2 0,0 0 0,0 0 0,0-2 0,-20-6 0,9 2 0,26 7 2,0 1 0,-1-1 0,1 1-1,0-1 1,0 0 0,0 1 0,0-1 0,0 0 0,0 0-1,0 0 1,0 0 0,1 0 0,-1 0 0,0 0-1,1 0 1,-1 0 0,0 0 0,1 0 0,-1-1-1,1 1 1,0 0 0,-1 0 0,1-1 0,0 1-1,0 0 1,0-2 0,0-39-274,1 24-870,-1 11-5684</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2591.65">185 955 24575,'298'0'-1365,"-292"0"-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3549.52">223 939 24575,'-5'1'0,"0"-1"0,-1 0 0,1 1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 1 0,0-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,0 1 0,-5 4 0,-14 7 0,-8 7 0,25-17-116,5-3 139,-1-1-1,1 0 1,0 1 0,-1-1 0,1 1-1,0-1 1,0 1 0,0 0 0,0 0-1,-1 2 1,2-3-70,0-1 0,0 1 1,1 0-1,-1 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 1,-1-1-1,1 1 0,-1 0 0,1-1 0,-1 1 0,1-1 1,-1 1-1,1 0 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 1 1,-1-1-1,1 0 0,0 1 0,0-1 0,0 0 0,-1 0 1,1 0-1,0 1 0,1-1 0,4 2-6779</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="5054.73">832 1412 24575,'-4'4'0,"1"1"0,-1 0 0,1 0 0,0 0 0,-5 11 0,-12 17 0,18-29 0,0 0 0,0 1 0,0-1 0,0 0 0,1 1 0,0-1 0,-2 7 0,-3 13 0,3-16 0,-1 1 0,0 1 0,1-1 0,0 1 0,0 0 0,1 0 0,1 0 0,-1 19 0,1-27 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,1 1 0,0-1 0,-1-1 0,1 1 0,2 1 0,14 16 0,-16-16 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1 0 0,2 1 0,32 18 0,-30-16 0,1 0 0,1-1 0,-1 1 0,0-2 0,13 5 0,12 7 0,-29-13 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,5 0 0,7 0 0,-9 0 0,-1 0 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1-1 0,12-3 0,-15 2 0,-1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,1-4 0,12-37 0,-12 34 0,-1-1 0,0 1 0,0 0 0,-1 0 0,0 0 0,-1 0 0,0-1 0,0 1 0,-4-12 0,0 16 0,0 0 0,0 1 0,-1-1 0,0 1 0,0 0 0,0 0 0,0 1 0,-1 0 0,0 0 0,0 1 0,-7-4 0,-45 1 0,35 4 0,6 2 0,0 0 0,1 1 0,-1 1 0,0 0 0,-27 9 0,35-9 0,-6 1 0,14-3 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 2 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,-1 2 0,-13 29-1365,14-26-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="6313.59">794 1457 24575,'8'0'16,"-1"-1"-1,0 0 0,1-1 0,-1 0 1,0 0-1,0 0 0,12-7 1,-12 6-202,-1 0 0,1 0 0,0 1 0,0-1 0,1 2 0,-1-1 0,11 0 0,-11 2-6640</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="7938.2">1114 1968 24575,'7'-3'0,"0"0"0,-1 0 0,2 1 0,-1 1 0,0-1 0,0 1 0,1 0 0,-1 1 0,0-1 0,9 2 0,-7-1 0,1 0 0,-1-1 0,0 0 0,0 0 0,0-1 0,15-5 0,-31 12 0,1-1 0,0 1 0,0 1 0,0-1 0,1 1 0,0 0 0,0 1 0,0-1 0,1 1 0,0 0 0,0 0 0,1 0 0,0 0 0,-4 12 0,7-15 0,-1-1 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-4 4 0,3-4 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,1-1 0,-2 3 0,-9 42 0,9-40 0,-1-1 0,1 1 0,1 0 0,-1 0 0,1 12 0,0-5-54,3 22-1257</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="8315.68">1030 2036 24575,'19'0'0,"-5"-1"0,-1 1 0,1 1 0,-1 0 0,0 1 0,24 6 0,-10-2-51,0 0-1,1-2 1,0-1-1,-1-1 1,48-3 0,-28 0-1006,-41 1-5769</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -13923,15 +14680,17 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:27.284"/>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-20T02:32:16.457"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
       <inkml:brushProperty name="width" value="0.035" units="cm"/>
       <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
     </inkml:brush>
   </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 0 24575</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">658 24 24575,'0'1'0,"0"1"0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 1 0,-1 0 0,0 0 0,1-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 2 0,1-2 0,-1 0 0,1 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 1 0,2 0 0,11 10 0,-9-5 0,1 0 0,-1 1 0,9 14 0,5 7 0,-7-11 0,0 0 0,11 21 0,-18-27 0,-1 1 0,0 0 0,-1 0 0,3 19 0,-7-30 0,1-1 0,-1 1 0,0-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 1 0,-1-1 0,-1 0 0,-10 1 0,1 0 0,-1-1 0,-18-1 0,12 0 0,7 1 0,4 0 0,-1 1 0,0-1 0,0-1 0,1 0 0,-1 0 0,0-1 0,1 0 0,-1 0 0,1-1 0,0 0 0,-12-6 0,-1 0 0,19 8 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,-2-2 0,1 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,0-1 0,0 0 0,-2-4 0,4 6 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1 0 0,0 0 0,3-2 0,0-1 0,0 0 0,1 1 0,-1-1 0,1 1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,1 1 0,-1-1 0,1 1 0,-1 0 0,9 0 0,-11 1 0,45-13 0,-39 10 0,1 0 0,0 0 0,14-2 0,-13 3 0,-1 0 0,0-1 0,0-1 0,16-8 0,-24 11 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1-3 0,-1-1 0,0 0 0,0 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,-7-8 0,1 1 0,-8-9 0,9 16 0,6 4 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-4-1 0,-76-7-1365,76 8-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1416">316 603 24575,'-7'-3'0,"1"0"0,-1 1 0,1 0 0,-1 0 0,0 1 0,0 0 0,0 0 0,0 1 0,-7 0 0,12-1 0,1 1 0,-6 0 0,-1-1 0,0 1 0,1 1 0,-1-1 0,-11 3 0,17-2 0,-1 0 0,0 0 0,1 1 0,-1-1 0,0 1 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 4 0,-47 78 0,47-80 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,3 6 0,-2-4 0,1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,1 0 0,0-1 0,0 1 0,0-1 0,1 0 0,5 3 0,7 5 0,-15-10 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,-1-1 0,6 2 0,-6-3 0,-1 0 0,1 1 0,-1-1 0,1-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,2-2 0,13-15 0,-14 15 0,0 0 0,1 1 0,-1-1 0,1 0 0,0 1 0,5-5 0,-4 5 0,-1-1 0,0 0 0,1 0 0,-1 0 0,-1-1 0,1 1 0,0-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1-6 0,-1 1 0,1-1 0,-1 1 0,-1-1 0,0 0 0,0 1 0,-3-15 0,3 22 0,0-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 1 0,-3-3 0,5 3 0,0 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,0 2 0,0-1 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 0 0,-1 1 0,1 1 0,-13 63 0,10-47 0,1-1 0,1 1 0,0 0 0,3 29 0,0 4 0,-1-41 0,-1-6 0,0 0 0,1 0 0,-1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,0 0 0,0-1 0,-1 1 0,-4 6 0,5-9 0,-1 1 0,0 0 0,0 0 0,0-1 0,0 0 0,-7 4 0,8-4 0,-1-1 0,0 1 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-2 4 0,2-5 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,-4 0 0,-11 0 0,-35-3 0,46 3 0,3-1-114,0 0 1,0 0-1,0-1 0,0 0 0,0 1 1,0-1-1,1 0 0,-1-1 0,1 1 1,-1-1-1,-3-3 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2214.56">856 1067 24575,'-10'11'0,"6"-7"0,1 0 0,-1-1 0,0 1 0,0-1 0,0 0 0,-1 0 0,-7 4 0,9-5 0,-1 1 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,1-1 0,-1 1 0,1 1 0,-2 5 0,-15 31 0,15-34 0,0 1 0,0 0 0,1 1 0,0-1 0,0 0 0,1 1 0,0-1 0,1 1 0,0 10 0,-1 0 0,1 110-1365,0-122-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2893.39">970 1158 24575,'-3'0'0,"-1"0"0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,1 1 0,-1-1 0,0 0 0,1 1 0,-1-1 0,1 1 0,0 0 0,0 0 0,0 0 0,-3 5 0,3-2 0,0-1 0,1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,1 0 0,0-1 0,0 1 0,0 0 0,1 0 0,0 0 0,0-1 0,4 11 0,-2-6 0,1 0 0,0-1 0,1 1 0,0-1 0,0 0 0,1 0 0,0 0 0,1-1 0,0 0 0,0 0 0,1 0 0,0-1 0,12 8 0,-11-8 0,-3-2 0,1 0 0,0-1 0,0 1 0,1-1 0,-1-1 0,9 4 0,-14-7 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,1-1 0,37-50 0,-36 45 0,0-1 0,-1 1 0,0-1 0,-1 0 0,0 1 0,0-1 0,-1 0 0,0 1 0,0-1 0,-3-12 0,1-15 0,2 31 0,-1 0 0,1 1 0,-1-1 0,-1 0 0,1 1 0,0-1 0,-1 0 0,0 1 0,0 0 0,-1-1 0,-2-3 0,-37-45 0,20 28 0,-13-9 77,29 29-318,-1-1 1,1 1 0,0-1 0,1 0-1,-9-12 1</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -13980,6 +14739,233 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-20T02:32:21.942"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">43 25 24575,'-7'161'0,"7"-104"0,1-49 0,-1-1 0,1 1 0,-1-1 0,0 1 0,-1-1 0,0 1 0,0-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,-5 10 0,-7 5-1365</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="749.97">149 93 24575,'0'-3'0,"0"-1"0,0 0 0,1 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,4-5 0,-3 8 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 1 0,3-1 0,17-7 0,-19 7 0,1-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,4 0 0,3-1 0,0 1 0,-1-2 0,19-3 0,-7 0 0,-19 4 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,4 2 0,-4-2 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,0-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,-1 3 0,0 18 0,1-15 0,0 0 0,0-1 0,-1 1 0,1 0 0,-2 0 0,1-1 0,-1 1 0,0-1 0,-6 12 0,3-7 0,0 0 0,-1 0 0,-1-1 0,0 0 0,0 0 0,-1-1 0,0 0 0,-1 0 0,-15 11 0,5-6 0,-35 30 0,37-36 0,31-9 0,247 1 0,-254-1-151,0 1-1,0-1 0,0-1 0,0 1 1,0-1-1,0-1 0,0 1 1,10-6-1</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink71.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-20T02:32:20.520"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">2 8 24575,'-1'0'0,"1"0"0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1-1 0,0 1 0,0 0 0,1 1 0,7 167 0,-7-115 0,-3 60 0,-9-75 103,4-18-1571,5-14-5358</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="576.52">146 54 24575,'1'13'0,"0"0"0,0 0 0,7 24 0,-6-28 0,1 12 0,0 1 0,-2 0 0,-1-1 0,-2 26 0,0 10 0,7 26 0,-8-67 0,3-16 0,0 1 0,-1 0 0,1 0 0,0-1 0,0 1 0,0 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,2 0 0,1 4-1365</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink72.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-20T02:32:23.793"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">32 1 24575,'0'18'0,"0"-8"0,1 0 0,-2 1 0,0-1 0,0 1 0,-1-1 0,-5 18 0,5-19 0,0 0 0,0 0 0,1-1 0,0 1 0,1 0 0,0 9 0,-2 33 0,0-43-109,-6 59-1147,8-61-5570</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="969">230 54 24575,'8'-1'0,"1"0"0,0 0 0,-1-1 0,15-5 0,-15 5 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1 0 0,12 0 0,-18 1 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-1 0 0,2 4 0,-2-5 0,0 1 0,0 0 0,-1 0 0,1 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,1 0 0,-3 0 0,-20 7 0,24-2 0,13 2 0,-3-4 0,-8-3 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,-1 0 0,1-1 0,1 3 0,-1-1 0,1 1 0,-1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0 3 0,-2-6 0,1 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-2-1 0,-135 8-1365,131-7-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink73.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-20T02:32:25.797"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 23 24575,'7'177'0,"-6"-117"-1365,-1-54-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="507.53">343 1 24575,'-1'5'0,"1"0"0,-1 1 0,0-1 0,0 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,-4 6 0,-10 30 0,12-29 0,0-1 0,0 0 0,-1-1 0,-12 21 0,4-17 0,11-12 0,-1 0 0,0 1 0,1 0 0,0-1 0,0 1 0,0 0 0,-3 4 0,5-6 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,-1 0 0,1 0 0,0 0 0,0 0 0,1 0 0,10 2 0,0 0 0,1-1 0,-1 0 0,1-1 0,22-2 0,8 0 0,-21 2 0,-14 1 0,-1-1 0,1 0 0,0 0 0,0-1 0,0 0 0,0 0 0,0-1 0,-1 0 0,13-5 0,-10 4 0,1-1 0,0 1 0,0 1 0,0 0 0,0 1 0,0 0 0,14 1 0,-3-1 0,-17 0-102,3 1-108,-1 0-1,1-1 1,-1 0-1,1-1 0,7-2 1,-7 1-6616</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="888.92">587 1 24575,'-1'8'0,"0"1"0,-1 0 0,1 0 0,-2-1 0,-4 15 0,3-15 0,1 1 0,1-1 0,0 1 0,0 0 0,0 0 0,1 10 0,0-14 0,1 0 0,-1-1 0,0 1 0,0 0 0,-3 8 0,-4 18 0,7-24 0,-1-1 0,0 1 0,0 0 0,0-1 0,-7 13 0,-6 17 0,-4 6-1365,18-36-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink74.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-20T02:32:30.663"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 115 24575,'0'191'-1365,"0"-185"-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="983.94">130 267 24575,'0'117'0,"0"-127"0,2 0 0,-1 0 0,1 0 0,1 1 0,0-1 0,0 0 0,1 1 0,0 0 0,1 0 0,0 0 0,0 0 0,10-11 0,-3-11 0,0-3 0,-11 33 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,2 0 0,-1 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,1 2 0,18 32 0,-4-6 0,-10-20 0,-1 1 0,-1-1 0,0 0 0,0 1 0,-1 0 0,0 0 0,-1 0 0,0 1 0,0-1 0,-1 16 0,1-10 0,-1-7 0,0-1 0,-1 1 0,0-1 0,0 1 0,-1-1 0,-3 16 0,4-23-62,-1 0 0,0 1 0,1-1 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1-1,0 0 1,0-1 0,0 1 0,0-1 0,0 1 0,-1-1 0,1 0 0,0 1 0,-2-1 0,-2 1-6764</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1772.33">122 130 24575,'1'-2'0,"-1"0"0,1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,0 0 0,-1 1 0,1-1 0,3-2 0,33-25 0,-29 22 0,-2 2 0,0 1 0,1-1 0,0 1 0,0 0 0,0 1 0,0 0 0,0 0 0,1 1 0,-1 0 0,12-1 0,7-9 0,-25 11 0,0-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1 1 0,1-1 0,0 0 0,0 1 0,3-1 0,47 2-1365,-46-1-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2505.57">76 100 24575,'0'16'0,"0"-6"0,-1 0 0,2 0 0,-1 0 0,1 0 0,1-1 0,0 1 0,0 0 0,1-1 0,5 14 0,8 30-1365</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink75.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:24.076"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 740 24575,'1'-8'5,"-1"1"1,1-1-1,0 0 0,0 1 0,1 0 0,-1-1 1,2 1-1,-1 0 0,1 0 0,0 0 0,0 0 1,1 1-1,-1-1 0,9-9 0,2 0-174,1 0 0,1 0 0,25-18 0,-25 22 95,0-1-1,-1-1 1,0-1-1,14-18 1,-14 10 74,-5 9 0,0 0 0,1 0 0,0 1 0,21-19 0,-22 22-6,1-1 0,-1 0 0,-1 0 0,0-1 0,-1-1 0,0 0 0,7-14 0,27-41 862,-37 62-830,0 0-1,1 1 0,0-1 0,0 2 1,0-1-1,13-6 0,-13 7-27,0 0 0,1 0 0,-1 0 1,-1-1-1,1 0 0,-1 0 0,9-11 0,1-12 2,-13 24 0,-1 0 0,1 0 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,0 1 0,0 0 0,0 0 0,5-3 0,-8 6 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,0 1 0,0 1 0,6 35 0,-6-35 0,3 385 0,-7-192 0,5 115-1365,-1-265-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink76.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:26.173"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 1 24575,'0'0'-8191</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink77.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:27.284"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 0 24575</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink78.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:35.128"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
@@ -13992,7 +14978,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink79.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -14017,233 +15003,6 @@
     </inkml:brush>
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1 24575,'748'0'-905,"-743"0"989,1 0 1,-1 0-1,0 1 0,0-1 1,0 1-1,0 0 0,0 1 1,0-1-1,0 1 0,5 2 0,-7-2-85,-1 0 0,1 1-1,0-1 1,-1 0 0,1 1-1,-1 0 1,0-1-1,0 1 1,0 0 0,0 0-1,-1 0 1,1 1-1,-1-1 1,0 0 0,2 6-1,23 46 2,-21-48 0,-1 1 0,0 0 0,0 0 0,-1 1 0,0-1 0,0 1 0,1 9 0,0 3 0,-1 1 0,-1 0 0,-1 0 0,-2 1 0,0-1 0,-1 0 0,-7 33 0,5-48 0,0 0 0,0 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1-1 0,0 0 0,-7 5 0,-30 31 0,23-19 0,-1-1 0,0-1 0,-2-2 0,0 0 0,-41 23 0,46-33 0,-1 0 0,0-2 0,0 0 0,0-1 0,-1-1 0,0-1 0,-26 1 0,-23 4 0,21-1 0,20-5 0,1 3 0,-32 8 0,53-12 0,0 1 0,0 0 0,0 0 0,1 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0 0 0,0 0 0,1 0 0,0 1 0,0 0 0,-5 6 0,9-10 0,0-1 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,0 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,34 5 0,-28-5 0,64 11 0,-30-4 0,74 4 0,-102-12 0,1 2 0,-1 0 0,0 0 0,1 1 0,-1 1 0,0 0 0,0 1 0,-1 0 0,1 1 0,-1 1 0,0 0 0,21 13 0,-19-10 0,-4-3 0,0 0 0,-1 0 0,1 1 0,-1 0 0,-1 0 0,1 1 0,-1 0 0,-1 1 0,0 0 0,10 15 0,-11-15 0,0 0 0,1 0 0,0-1 0,0 0 0,1 0 0,0-1 0,1 0 0,11 8 0,-10-7 0,1-1 0,-2 2 0,1-1 0,-1 1 0,-1 1 0,9 11 0,7 22 0,-1 1 0,-3 0 0,-1 2 0,-2 0 0,10 49 0,-22-80 0,0-1 0,1 0 0,11 17 0,7 18 0,-20-41 0,1 0 0,-1 0 0,1 0 0,9 9 0,-10-12 0,0 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1 0 0,-1 0 0,1 1 0,-1-1 0,2 8 0,-4-10 0,1 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0-1 0,-1 0 0,1 0 0,-1 1 0,1-2 0,-1 1 0,0 0 0,0 0 0,0-1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,0 0 0,1 0 0,-1-1 0,0 0 0,0 0 0,-6 1 0,-16 3 0,0-2 0,0 0 0,0-2 0,-41-3 0,35 0 0,-468 1 0,476 2 43,0 2-1,-38 8 0,-12 2-1534,47-11-5334</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink72.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:49.542"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">477 1 24575,'0'16'0,"0"1"0,-1 0 0,-1 0 0,-1-1 0,0 1 0,-1-1 0,-1 0 0,-1 0 0,0 0 0,-1-1 0,-1 0 0,0 0 0,-1-1 0,-17 21 0,5-7 0,1 1 0,1 0 0,2 1 0,-20 48 0,26-57 0,-1 0 0,-1-1 0,-1-1 0,-1 0 0,-22 23 0,13-15 0,17-18 0,0 1 0,1 0 0,0 0 0,1 1 0,0 0 0,1 0 0,-5 16 0,6-16 0,-1 0 0,0 0 0,0 0 0,-1 0 0,-1-1 0,0 0 0,-14 18 0,14-22 0,1 0 0,0 1 0,1-1 0,-1 1 0,1 0 0,1 1 0,-1-1 0,1 0 0,1 1 0,-1 0 0,0 8 0,3-15 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,3-1 0,49 2 0,-44-1 0,837-4-1123,-651 4 279,-168 0-5380</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="437.97">978 513 24575,'0'0'0,"0"-1"0,1 0 0,-1 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,1 1 0,-2 0 0,-2 0 0,1 1 0,-1 0 0,0 0 0,0 1 0,1-1 0,0 1 0,-6 4 0,-126 170 0,79-100 0,8 4 0,24-35 0,15-27 0,1 0 0,1 1 0,0 0 0,-4 25 0,-12 36 0,-1-10 0,3 1 0,-16 98 0,35-159 15,-2 0 0,0 0-1,0 0 1,-1 0 0,0-1 0,-1 0-1,-9 12 1,-18 36-1498,24-35-5343</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink73.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:52.121"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">265 382 24575,'-31'182'0,"30"-171"0,0 1 0,-2 0 0,1-1 0,-1 0 0,-1 0 0,0 0 0,-1 0 0,0 0 0,0-1 0,-1 0 0,-1 0 0,0-1 0,-13 15 0,-30 45 0,27-36 0,-42 46 0,64-78 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,1 3 0,0-2 0,0-1 0,0 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 0 0,2 0 0,10 2 0,-1-2 0,1 1 0,-1-2 0,1 0 0,13-3 0,161-23 0,-154 24 0,22-9 0,-43 8 0,0 1 0,-1 1 0,1 0 0,19 0 0,-28 2 0,0 0 0,0 1 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 1 0,3 5 0,0 1 0,0 1 0,-1 0 0,0-1 0,-1 2 0,4 12 0,-6-15 0,0-1 0,0 0 0,1 1 0,1-1 0,-1 0 0,1 0 0,0-1 0,0 1 0,1-1 0,0 0 0,9 8 0,-8-8 0,0 0 0,0 1 0,-1-1 0,0 1 0,0 0 0,0 1 0,6 13 0,-7-11 0,1-1 0,1 1 0,0-1 0,13 14 0,-15-18 0,1-1 0,-1 0 0,0 1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,-1 0 0,-1 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,-1 0 0,0 7 0,-1-3 0,-1 0 0,-1-1 0,0 1 0,0-1 0,-1 0 0,0 0 0,0 0 0,-1 0 0,0-1 0,-9 11 0,-57 72 0,42-56 0,25-28 0,-1 0 0,0-1 0,0 0 0,0 0 0,-1 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,0-1 0,0 0 0,0 0 0,-11 4 0,-22 2 0,26-7 0,0 0 0,0 0 0,0 2 0,1-1 0,0 2 0,0 0 0,0 0 0,1 1 0,0 1 0,-19 15 0,25-18 0,0 0 0,-1 0 0,0 0 0,0-1 0,0 0 0,0 0 0,0-1 0,-1 0 0,0 0 0,1-1 0,-1 0 0,0 0 0,0-1 0,-15 1 0,-7-1 0,0-1 0,-48-6 0,73 5-105,0 0 0,0 0 0,0-1 0,0 1 0,0-1 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 0 0,-4-4 0,-6-5-6721</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="443">370 1 24575,'14'2'0,"1"0"0,0 1 0,-1 1 0,0 1 0,0 0 0,0 0 0,-1 2 0,24 13 0,-21-11 0,9 5 0,0-1 0,0-1 0,2-1 0,-1-2 0,1 0 0,0-2 0,1-1 0,0-1 0,48 2 0,939-10-1493,-989 3-5205</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink74.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:06:10.193"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1253 1 24575,'-35'0'0,"-1"2"0,1 1 0,0 1 0,-61 17 0,82-17 0,1 0 0,0 1 0,0 1 0,1 0 0,0 1 0,0 0 0,0 0 0,1 1 0,0 1 0,1 0 0,0 1 0,0 0 0,1 0 0,0 1 0,-8 13 0,9-12 0,-1 0 0,-1-1 0,1 0 0,-2 0 0,-14 11 0,12-11 0,0 1 0,1 0 0,-14 19 0,0 4 0,17-25 0,1 1 0,0 0 0,1 0 0,0 1 0,0 0 0,1 1 0,1-1 0,-4 17 0,6-22 0,0 1 0,-1-1 0,1 0 0,-1 0 0,-1 0 0,1 0 0,-1-1 0,-11 11 0,9-8 0,0 0 0,0 0 0,-10 17 0,9-9 0,0-1 0,2 1 0,0 0 0,-4 20 0,9-31 0,0 1 0,0 0 0,0-1 0,1 1 0,0 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,1 1 0,0-1 0,1 1 0,3 5 0,37 56 0,-32-54 0,-2 1 0,1 0 0,-2 0 0,0 1 0,-1 0 0,6 18 0,-11-30 0,0 1 0,0 0 0,0-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1-1 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0-1 0,1 0 0,0 0 0,0 0 0,-1-1 0,6 1 0,15 4 0,-1-1 0,1-2 0,27 1 0,-49-4 0,2 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,0 0 0,0 1 0,-1-2 0,1 1 0,-1 0 0,1-1 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,-1-1 0,1 1 0,0-6 0,22-45 0,-18 43 0,0 0 0,-1 0 0,-1 0 0,0-1 0,0 1 0,2-17 0,-6 26 0,0-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-4 0 0,-7-3 0,1 1 0,-1 0 0,-1 0 0,1 2 0,-1 0 0,-18-1 0,-94 6 0,55 0 0,12-2 0,-1 2 0,-66 13 0,-65 16 0,121-23 65,51-8-541,0 2-1,-37 8 0,38-4-6349</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink75.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:06:11.362"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 192 24575,'1'-2'0,"-1"-1"0,1 1 0,0-1 0,0 0 0,0 1 0,0 0 0,0-1 0,0 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,1 0 0,2-2 0,57-25 0,-51 24 0,9-5 0,0-1 0,0-1 0,31-23 0,-26 16 0,-17 14 0,-1 0 0,1 0 0,0 0 0,0 1 0,0 1 0,1-1 0,-1 1 0,0 1 0,13-1 0,-1 0 0,0 2 0,37 4 0,-54-4 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,2 4 0,-1 0 0,0 0 0,0 0 0,-1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,0 7 0,-1 0 0,0-1 0,0 1 0,-1-1 0,-1 1 0,0-1 0,-1 0 0,0 0 0,0 0 0,-10 19 0,-28 34 0,32-55 0,1 1 0,1 0 0,0 1 0,1-1 0,0 1 0,0 1 0,2-1 0,-1 1 0,2 0 0,-1 0 0,0 14 0,4 109-23,1-85-1319,0-24-5484</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="560.65">187 529 24575,'0'-3'0,"0"0"0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 1 0,4-2 0,12-1 0,-1 0 0,1 1 0,29 0 0,0 0 0,145-15-527,-80 9 296,-19-6 231,-61 8 0,55-4 0,-54 8 394,52-11-1,-10 1-1787,-51 10-5432</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink76.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:06:13.299"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1 24575,'0'0'-8191</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink77.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:23.923"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 560 24575,'1'-1'0,"0"1"0,1-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1-1 0,1-1 0,15-37 0,-12 28 0,21-60 0,16-80 0,-22 75 0,-16 69 0,0 1 0,1-1 0,0 0 0,0 1 0,1 0 0,-1 0 0,2 0 0,-1 1 0,1-1 0,0 1 0,0 1 0,7-6 0,-4 4 0,0-1 0,-1 0 0,-1-1 0,1 1 0,11-20 0,-18 27 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 1 0,0-1 0,2 0 0,-3 2 0,1-1 0,0 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1-1 0,0 1 0,0 0 0,0 1 0,6 59 0,-6-51 0,0 1 0,-1-1 0,0 1 0,-1-1 0,0 0 0,0 1 0,-1-1 0,0-1 0,-1 1 0,-6 12 0,3-6 0,1 0 0,1 1 0,1 0 0,0 0 0,1 0 0,-1 30 0,2-28 0,0 0 0,-1 0 0,-1 0 0,0 0 0,-10 24 0,-50 134 0,12-30 0,49-141 0,0-1 0,0 1 0,-1-1 0,0 1 0,-7 7 0,-15 22 0,17-19-1365,0-3-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink78.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:25.843"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 2 24575,'85'-1'0,"96"3"0,-176-1 0,1 0 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,0 0 0,-1 0 0,1 0 0,8 8 0,43 48 0,-47-48 0,1 5 0,-1 0 0,0 1 0,-1 0 0,-1 1 0,-1-1 0,8 35 0,-10-35 0,17 53 0,17 67 0,-37-125 0,0-1 0,-1 1 0,0-1 0,-1 1 0,0-1 0,-1 0 0,0 1 0,0-1 0,-2 0 0,1 0 0,-1 0 0,-6 10 0,0-2 0,0-1 0,-1 0 0,-1-1 0,-1 0 0,-27 27 0,-6-6 0,36-30 0,0-1 0,0 2 0,1-1 0,0 1 0,-10 14 0,16-18 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1-1 0,0 0 0,-1 0 0,1 0 0,-1-1 0,1 0 0,-10 0 0,121 0 0,174-4 0,-270 2 0,0 0 0,0 0 0,0-1 0,-1-1 0,1 1 0,10-7 0,-11 6 0,1-1 0,0 1 0,1 1 0,-1-1 0,20-2 0,148 4 63,-93 4-1491,-62-2-5398</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink79.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:29.383"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">487 32 24575,'0'-2'0,"1"1"0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,3 0 0,42-5 0,-41 5 0,18-2 0,-8 0 0,1 1 0,-1 1 0,0 0 0,29 4 0,-42-2 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 4 0,1 12 0,0 1 0,-2 26 0,0-31 0,-1-6 0,0 0 0,0 0 0,-1-1 0,0 1 0,0 0 0,-1 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,-1 0 0,0-1 0,0 1 0,-1-1 0,0 0 0,0 0 0,-1-1 0,-11 9 0,-8 4 0,-1-1 0,-1-2 0,-59 26 0,71-34 0,0 2 0,1-1 0,-17 15 0,20-15 0,0 0 0,-1 0 0,0-1 0,-1 0 0,-14 5 0,-4-1 0,0-2 0,0-1 0,-37 5 0,62-13 0,1 0 0,0 1 0,0 0 0,0 0 0,0 0 0,0 1 0,1 0 0,-1 0 0,1 0 0,-1 1 0,-7 7 0,12-11 0,1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,2 1 0,29 3 0,-30-3 0,5 0 0,38 2 0,60-5 0,-89 1 0,-1 0 0,0-1 0,0 0 0,0-1 0,0-1 0,0 0 0,-1 0 0,14-9 0,-10 4 0,-1 1 0,1 1 0,1 1 0,-1 0 0,1 1 0,0 1 0,1 1 0,-1 0 0,1 1 0,0 1 0,29 0 0,-45 3 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1-1 0,0 2 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 5 0,1 13 0,-1 0 0,-1-1 0,-4 32 0,1-16 0,3 13 0,0-20 0,-1-1 0,-6 31 0,5-49 0,0-1 0,-1 1 0,0-1 0,0 0 0,-1 0 0,0 0 0,-1-1 0,0 1 0,-1-1 0,-6 7 0,-17 28 0,25-37 0,0 1 0,0-1 0,0 0 0,-1 0 0,0 0 0,0 0 0,-1-1 0,0 0 0,-11 8 0,-7 2 0,0-1 0,-1 0 0,0-2 0,-1-1 0,-1-1 0,0-2 0,0 0 0,-55 8 0,68-14 0,-1 1 0,0 1 0,1 0 0,-17 8 0,17-6 0,0-1 0,0-1 0,0 0 0,-27 4 0,-34-2-1365,57 0-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -14291,6 +15050,233 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:49.542"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">477 1 24575,'0'16'0,"0"1"0,-1 0 0,-1 0 0,-1-1 0,0 1 0,-1-1 0,-1 0 0,-1 0 0,0 0 0,-1-1 0,-1 0 0,0 0 0,-1-1 0,-17 21 0,5-7 0,1 1 0,1 0 0,2 1 0,-20 48 0,26-57 0,-1 0 0,-1-1 0,-1-1 0,-1 0 0,-22 23 0,13-15 0,17-18 0,0 1 0,1 0 0,0 0 0,1 1 0,0 0 0,1 0 0,-5 16 0,6-16 0,-1 0 0,0 0 0,0 0 0,-1 0 0,-1-1 0,0 0 0,-14 18 0,14-22 0,1 0 0,0 1 0,1-1 0,-1 1 0,1 0 0,1 1 0,-1-1 0,1 0 0,1 1 0,-1 0 0,0 8 0,3-15 0,1 0 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,3-1 0,49 2 0,-44-1 0,837-4-1123,-651 4 279,-168 0-5380</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="437.97">978 513 24575,'0'0'0,"0"-1"0,1 0 0,-1 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,1 1 0,-2 0 0,-2 0 0,1 1 0,-1 0 0,0 0 0,0 1 0,1-1 0,0 1 0,-6 4 0,-126 170 0,79-100 0,8 4 0,24-35 0,15-27 0,1 0 0,1 1 0,0 0 0,-4 25 0,-12 36 0,-1-10 0,3 1 0,-16 98 0,35-159 15,-2 0 0,0 0-1,0 0 1,-1 0 0,0-1 0,-1 0-1,-9 12 1,-18 36-1498,24-35-5343</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink81.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:05:52.121"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">265 382 24575,'-31'182'0,"30"-171"0,0 1 0,-2 0 0,1-1 0,-1 0 0,-1 0 0,0 0 0,-1 0 0,0 0 0,0-1 0,-1 0 0,-1 0 0,0-1 0,-13 15 0,-30 45 0,27-36 0,-42 46 0,64-78 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,1 3 0,0-2 0,0-1 0,0 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,-1 1 0,1-1 0,0 0 0,2 0 0,10 2 0,-1-2 0,1 1 0,-1-2 0,1 0 0,13-3 0,161-23 0,-154 24 0,22-9 0,-43 8 0,0 1 0,-1 1 0,1 0 0,19 0 0,-28 2 0,0 0 0,0 1 0,-1-1 0,1 1 0,0 0 0,-1 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 1 0,3 5 0,0 1 0,0 1 0,-1 0 0,0-1 0,-1 2 0,4 12 0,-6-15 0,0-1 0,0 0 0,1 1 0,1-1 0,-1 0 0,1 0 0,0-1 0,0 1 0,1-1 0,0 0 0,9 8 0,-8-8 0,0 0 0,0 1 0,-1-1 0,0 1 0,0 0 0,0 1 0,6 13 0,-7-11 0,1-1 0,1 1 0,0-1 0,13 14 0,-15-18 0,1-1 0,-1 0 0,0 1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,-1 0 0,-1 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,-1 0 0,0 7 0,-1-3 0,-1 0 0,-1-1 0,0 1 0,0-1 0,-1 0 0,0 0 0,0 0 0,-1 0 0,0-1 0,-9 11 0,-57 72 0,42-56 0,25-28 0,-1 0 0,0-1 0,0 0 0,0 0 0,-1 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,0-1 0,0 0 0,0 0 0,-11 4 0,-22 2 0,26-7 0,0 0 0,0 0 0,0 2 0,1-1 0,0 2 0,0 0 0,0 0 0,1 1 0,0 1 0,-19 15 0,25-18 0,0 0 0,-1 0 0,0 0 0,0-1 0,0 0 0,0 0 0,0-1 0,-1 0 0,0 0 0,1-1 0,-1 0 0,0 0 0,0-1 0,-15 1 0,-7-1 0,0-1 0,-48-6 0,73 5-105,0 0 0,0 0 0,0-1 0,0 1 0,0-1 0,1 0 0,-1-1 0,1 1 0,-1-1 0,1 0 0,0 0 0,-4-4 0,-6-5-6721</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="443">370 1 24575,'14'2'0,"1"0"0,0 1 0,-1 1 0,0 1 0,0 0 0,0 0 0,-1 2 0,24 13 0,-21-11 0,9 5 0,0-1 0,0-1 0,2-1 0,-1-2 0,1 0 0,0-2 0,1-1 0,0-1 0,48 2 0,939-10-1493,-989 3-5205</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink82.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:06:10.193"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1253 1 24575,'-35'0'0,"-1"2"0,1 1 0,0 1 0,-61 17 0,82-17 0,1 0 0,0 1 0,0 1 0,1 0 0,0 1 0,0 0 0,0 0 0,1 1 0,0 1 0,1 0 0,0 1 0,0 0 0,1 0 0,0 1 0,-8 13 0,9-12 0,-1 0 0,-1-1 0,1 0 0,-2 0 0,-14 11 0,12-11 0,0 1 0,1 0 0,-14 19 0,0 4 0,17-25 0,1 1 0,0 0 0,1 0 0,0 1 0,0 0 0,1 1 0,1-1 0,-4 17 0,6-22 0,0 1 0,-1-1 0,1 0 0,-1 0 0,-1 0 0,1 0 0,-1-1 0,-11 11 0,9-8 0,0 0 0,0 0 0,-10 17 0,9-9 0,0-1 0,2 1 0,0 0 0,-4 20 0,9-31 0,0 1 0,0 0 0,0-1 0,1 1 0,0 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,1 1 0,0-1 0,1 1 0,3 5 0,37 56 0,-32-54 0,-2 1 0,1 0 0,-2 0 0,0 1 0,-1 0 0,6 18 0,-11-30 0,0 1 0,0 0 0,0-1 0,1 0 0,0 1 0,0-1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1-1 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,0-1 0,1 0 0,0 0 0,0 0 0,-1-1 0,6 1 0,15 4 0,-1-1 0,1-2 0,27 1 0,-49-4 0,2 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,0 0 0,0 1 0,-1-2 0,1 1 0,-1 0 0,1-1 0,-1 1 0,0-1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,-1-1 0,1 1 0,0-6 0,22-45 0,-18 43 0,0 0 0,-1 0 0,-1 0 0,0-1 0,0 1 0,2-17 0,-6 26 0,0-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-4 0 0,-7-3 0,1 1 0,-1 0 0,-1 0 0,1 2 0,-1 0 0,-18-1 0,-94 6 0,55 0 0,12-2 0,-1 2 0,-66 13 0,-65 16 0,121-23 65,51-8-541,0 2-1,-37 8 0,38-4-6349</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink83.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:06:11.362"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 192 24575,'1'-2'0,"-1"-1"0,1 1 0,0-1 0,0 0 0,0 1 0,0 0 0,0-1 0,0 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,1 0 0,2-2 0,57-25 0,-51 24 0,9-5 0,0-1 0,0-1 0,31-23 0,-26 16 0,-17 14 0,-1 0 0,1 0 0,0 0 0,0 1 0,0 1 0,1-1 0,-1 1 0,0 1 0,13-1 0,-1 0 0,0 2 0,37 4 0,-54-4 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,0-1 0,2 4 0,-1 0 0,0 0 0,0 0 0,-1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,0 7 0,-1 0 0,0-1 0,0 1 0,-1-1 0,-1 1 0,0-1 0,-1 0 0,0 0 0,0 0 0,-10 19 0,-28 34 0,32-55 0,1 1 0,1 0 0,0 1 0,1-1 0,0 1 0,0 1 0,2-1 0,-1 1 0,2 0 0,-1 0 0,0 14 0,4 109-23,1-85-1319,0-24-5484</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="560.65">187 529 24575,'0'-3'0,"0"0"0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 1 0,4-2 0,12-1 0,-1 0 0,1 1 0,29 0 0,0 0 0,145-15-527,-80 9 296,-19-6 231,-61 8 0,55-4 0,-54 8 394,52-11-1,-10 1-1787,-51 10-5432</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink84.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:06:13.299"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1 24575,'0'0'-8191</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink85.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:23.923"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 560 24575,'1'-1'0,"0"1"0,1-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1-1 0,1-1 0,15-37 0,-12 28 0,21-60 0,16-80 0,-22 75 0,-16 69 0,0 1 0,1-1 0,0 0 0,0 1 0,1 0 0,-1 0 0,2 0 0,-1 1 0,1-1 0,0 1 0,0 1 0,7-6 0,-4 4 0,0-1 0,-1 0 0,-1-1 0,1 1 0,11-20 0,-18 27 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,0 1 0,0-1 0,2 0 0,-3 2 0,1-1 0,0 0 0,-1 1 0,1-1 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0 0 0,1 0 0,-1-1 0,0 1 0,0 0 0,0 1 0,6 59 0,-6-51 0,0 1 0,-1-1 0,0 1 0,-1-1 0,0 0 0,0 1 0,-1-1 0,0-1 0,-1 1 0,-6 12 0,3-6 0,1 0 0,1 1 0,1 0 0,0 0 0,1 0 0,-1 30 0,2-28 0,0 0 0,-1 0 0,-1 0 0,0 0 0,-10 24 0,-50 134 0,12-30 0,49-141 0,0-1 0,0 1 0,-1-1 0,0 1 0,-7 7 0,-15 22 0,17-19-1365,0-3-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink86.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:25.843"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 2 24575,'85'-1'0,"96"3"0,-176-1 0,1 0 0,-1 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,0 0 0,-1 0 0,1 0 0,8 8 0,43 48 0,-47-48 0,1 5 0,-1 0 0,0 1 0,-1 0 0,-1 1 0,-1-1 0,8 35 0,-10-35 0,17 53 0,17 67 0,-37-125 0,0-1 0,-1 1 0,0-1 0,-1 1 0,0-1 0,-1 0 0,0 1 0,0-1 0,-2 0 0,1 0 0,-1 0 0,-6 10 0,0-2 0,0-1 0,-1 0 0,-1-1 0,-1 0 0,-27 27 0,-6-6 0,36-30 0,0-1 0,0 2 0,1-1 0,0 1 0,-10 14 0,16-18 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1-1 0,-1 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1-1 0,0 0 0,-1 0 0,1 0 0,-1-1 0,1 0 0,-10 0 0,121 0 0,174-4 0,-270 2 0,0 0 0,0 0 0,0-1 0,-1-1 0,1 1 0,10-7 0,-11 6 0,1-1 0,0 1 0,1 1 0,-1-1 0,20-2 0,148 4 63,-93 4-1491,-62-2-5398</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink87.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:29.383"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">487 32 24575,'0'-2'0,"1"1"0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,3 0 0,42-5 0,-41 5 0,18-2 0,-8 0 0,1 1 0,-1 1 0,0 0 0,29 4 0,-42-2 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 1 0,1-1 0,-1 1 0,0 0 0,0-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 4 0,1 12 0,0 1 0,-2 26 0,0-31 0,-1-6 0,0 0 0,0 0 0,-1-1 0,0 1 0,0 0 0,-1 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,-1 0 0,0-1 0,0 1 0,-1-1 0,0 0 0,0 0 0,-1-1 0,-11 9 0,-8 4 0,-1-1 0,-1-2 0,-59 26 0,71-34 0,0 2 0,1-1 0,-17 15 0,20-15 0,0 0 0,-1 0 0,0-1 0,-1 0 0,-14 5 0,-4-1 0,0-2 0,0-1 0,-37 5 0,62-13 0,1 0 0,0 1 0,0 0 0,0 0 0,0 0 0,0 1 0,1 0 0,-1 0 0,1 0 0,-1 1 0,-7 7 0,12-11 0,1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0-1 0,2 1 0,29 3 0,-30-3 0,5 0 0,38 2 0,60-5 0,-89 1 0,-1 0 0,0-1 0,0 0 0,0-1 0,0-1 0,0 0 0,-1 0 0,14-9 0,-10 4 0,-1 1 0,1 1 0,1 1 0,-1 0 0,1 1 0,0 1 0,1 1 0,-1 0 0,1 1 0,0 1 0,29 0 0,-45 3 0,0-1 0,0 1 0,0 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,-1 0 0,1 0 0,-1-1 0,0 2 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 5 0,1 13 0,-1 0 0,-1-1 0,-4 32 0,1-16 0,3 13 0,0-20 0,-1-1 0,-6 31 0,5-49 0,0-1 0,-1 1 0,0-1 0,0 0 0,-1 0 0,0 0 0,-1-1 0,0 1 0,-1-1 0,-6 7 0,-17 28 0,25-37 0,0 1 0,0-1 0,0 0 0,-1 0 0,0 0 0,0 0 0,-1-1 0,0 0 0,-11 8 0,-7 2 0,0-1 0,-1 0 0,0-2 0,-1-1 0,-1-1 0,0-2 0,0 0 0,-55 8 0,68-14 0,-1 1 0,0 1 0,1 0 0,-17 8 0,17-6 0,0-1 0,0-1 0,0 0 0,-27 4 0,-34-2-1365,57 0-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink88.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:34.934"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
@@ -14304,7 +15290,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink81.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink89.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -14330,235 +15316,6 @@
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">49 96 24575,'0'50'0,"1"10"0,-2-1 0,-14 92 0,10-128 0,2-9 0,0 1 0,1 0 0,0 0 0,1 19 0,1-33 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,0-1 0,0 1 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,0 0 0,0 0 0,2 0 0,38 0 0,-32 0 0,58-3 0,0-1 0,83 7 0,-145-2 0,0 0 0,0 0 0,0 0 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,0 0 0,5 7 0,-6-8 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 1 0,0 0 0,1-1 0,-1 1 0,0 0 0,-1 0 0,1-1 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,0 1 0,0 0 0,0 0 0,0-1 0,-3 7 0,-2 2 0,0-1 0,-1 0 0,0 0 0,-1 0 0,0-1 0,-1 0 0,1-1 0,-13 10 0,-5 7 0,22-21 0,0-1 0,0 0 0,0 1 0,-1-1 0,1-1 0,-1 1 0,-6 3 0,-2-1 8,-1-1 0,0 0 0,0-1-1,0 0 1,0-1 0,-21 2 0,-88-5-330,66-1-776,35 1-5728</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="813.55">160 186 24575,'0'-3'0,"0"-1"0,0 1 0,0-1 0,0 1 0,1-1 0,0 1 0,-1 0 0,1-1 0,0 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,0 0 0,-1 0 0,4-2 0,-2 2 0,0 1 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 1 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,-1 0 0,9 0 0,30-1 0,-31 2 0,0-1 0,0 1 0,-1-2 0,1 0 0,0 0 0,-1-1 0,13-5 0,-5 1 0,-1 2 0,0 0 0,1 0 0,0 2 0,0 0 0,0 1 0,23 2 0,12-3 0,-29 0 39,0-2 0,41-13 0,-43 11-410,0 1 1,1 1-1,25-2 1,-27 6-6456</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink82.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:42.481"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">420 0 24575,'-6'0'0,"1"1"0,0-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 1 0,0 1 0,0-1 0,0 1 0,1 0 0,-1 0 0,1 0 0,0 0 0,-6 7 0,1 1 0,1 0 0,0 0 0,1 0 0,1 1 0,-11 25 0,8-20 0,0-1 0,-1 0 0,-1-1 0,-23 28 0,-24 33 0,28-21 0,-24 62 0,38-81 0,11-18 0,0 0 0,1 1 0,1-1 0,1 1 0,0 0 0,2 0 0,0 0 0,3 22 0,-1 14 0,-2-52 0,0 1 0,0-1 0,0 1 0,0-1 0,1 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,4 4 0,-1-3 0,0-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,-1 0 0,1 0 0,-1-1 0,1 1 0,10-2 0,333-4 0,-342 5 0,-1-1 0,0 1 0,0-1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,1 0 0,4-4 0,5-5 0,-2-1 0,1 0 0,13-18 0,-20 20 0,-1 1 0,0-2 0,0 1 0,-1-1 0,-1 0 0,0 0 0,-1 0 0,0 0 0,0-1 0,0-15 0,-3 26 0,0 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,-3-1 0,-57-22 0,33 15 0,-4-5 0,-1 0 0,-1 3 0,0 1 0,-1 1 0,0 2 0,0 1 0,-45 0 0,57 6 0,-1-1 0,1-1 0,-46-9 0,2 1-1365,46 9-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink83.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:51.648"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 106 24575,'54'-20'0,"67"10"0,-81 8 0,53-8 0,109-17 0,-117 16 0,19-4 0,-101 14 0,48-8 0,-49 9 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,2 2 0,-3-1 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-3 3 0,-22 36 0,18-31 0,-1 6 0,0 1 0,1 0 0,0 1 0,2-1 0,0 1 0,1 0 0,-3 24 0,2-12 0,-13 44 0,4-14 0,13-51 0,-1 0 0,1 0 0,-2 0 0,1 0 0,-1 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,-7 9 0,7-13 0,1 0 0,-1 1 0,1 0 0,0 0 0,0 0 0,-4 9 0,6-11 0,1 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,2 4 0,-2-3 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 1 0,-1 2 0,-21 48 0,18-45 0,0 1 0,0-1 0,1 1 0,-3 13 0,-45 162-1365,49-166-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="449.47">31 314 24575,'894'0'0,"-877"-1"19,1-1 0,33-8 0,-11 1-1441,-18 6-5404</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink84.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:53.534"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">111 1 24575,'0'12'0,"2"0"0,-1 0 0,2 0 0,-1 0 0,2 0 0,0-1 0,0 1 0,1-1 0,1 0 0,0 0 0,0-1 0,2 0 0,8 11 0,-1 3 0,-1 1 0,-2 0 0,12 32 0,-10-23 0,7 36 0,-19-59 0,0 1 0,1-1 0,1 0 0,0 0 0,1 0 0,0-1 0,1 0 0,10 15 0,-3-11 0,-1 0 0,-1 0 0,-1 1 0,0 1 0,-1-1 0,0 1 0,8 25 0,-10-21 0,1-1 0,0 0 0,22 31 0,-22-37 0,1 0 0,-2 0 0,0 1 0,-1-1 0,-1 1 0,0 1 0,-1-1 0,4 26 0,-6-18 0,0 6 0,-2 0 0,-2 34 0,1-56 0,0-1 0,1 1 0,-2 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,0-1 0,0 1 0,0-1 0,-8 7 0,6-8 0,0 1 0,0-2 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,0-1 0,-12 0 0,-79-4 0,49 0 0,13 4 0,22-1 0,-1 0 0,0 0 0,0-2 0,-24-4 0,34 5 0,0 0 0,1-1 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,1-2 0,0 1 0,-1 0 0,1-1 0,1 1 0,-1-1 0,0 0 0,-2-6 0,-2-1 0,2 0 0,-1 0 0,1 0 0,1-1 0,0 1 0,1-1 0,0 0 0,1 0 0,1 0 0,0 0 0,0 0 0,2 0 0,-1 0 0,2 0 0,4-18 0,7-6 0,2 2 0,21-36 0,-10 22 0,-19 37 0,1 0 0,0 1 0,1 0 0,0 1 0,1-1 0,0 2 0,23-16 0,17-16 0,-24 16 0,-13 11 0,1 0 0,0 0 0,1 1 0,1 1 0,0 0 0,1 1 0,20-9 0,-18 10 0,1-2 0,-1 0 0,-1-1 0,20-16 0,-5 4 0,-25 19 0,0 0 0,0 1 0,1 0 0,-1 1 0,1 0 0,11-3 0,-12 4 0,0 0 0,0 0 0,0-1 0,-1 0 0,0-1 0,0 1 0,0-1 0,10-7 0,83-57 0,-99 67-40,1-1 0,-1 1 0,0-1 0,1 1-1,-1-1 1,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 0-1,-1 0 1,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0-1,0 0 1,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,0-1-1,1 0 1,-1 0 0,0 0 0,0 0 0,0 1 0,0-1-1,0 0 1,0 1 0,-2-3 0,-7-11-6786</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink85.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:54.983"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1901 74 24575,'-653'0'0,"626"-1"0,1-2 0,-31-6 0,29 4 0,1 1 0,-28-1 0,-370 6 0,409 1 0,1 1 0,-1 0 0,1 1 0,0 1 0,0 0 0,0 1 0,1 1 0,-25 15 0,-6 1 0,35-17 0,0 1 0,1 0 0,-1 0 0,1 0 0,1 1 0,0 1 0,0 0 0,0 0 0,1 0 0,-7 13 0,-33 38 0,39-51 0,1 0 0,1 0 0,0 1 0,0 0 0,1 0 0,0 0 0,1 0 0,0 1 0,0 0 0,1 0 0,1 0 0,-2 12 0,0 17 0,3 82 0,2-84 0,-2-34 0,1 0 0,1 0 0,-1 1 0,0-1 0,1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 0 0,3 4 0,1-2 0,0-1 0,0 1 0,1-1 0,0-1 0,-1 1 0,1-1 0,16 4 0,10 1 0,0-2 0,0 0 0,65 0 0,105-13 0,-178 6 0,0-3 0,29-6 0,-46 8 0,1-1 0,-1 0 0,0 0 0,0-1 0,0-1 0,-1 1 0,1-2 0,-1 1 0,8-7 0,59-44 0,-17 14 0,-50 36 0,6-4 0,-1-2 0,0 0 0,16-17 0,-25 23 0,1-1 0,-1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,-1-1 0,0 1 0,0 0 0,1-12 0,20-167 0,-11 112 0,-7 48 0,-1 0 0,0-33 0,-3 44 0,-1 10 0,1 0 0,-1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,-3-7 0,4 11 0,0 1 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 0 0,-1 2 0,-18 25 0,16-22 0,-87 145 0,81-132 0,1 0 0,1 1 0,0 0 0,2 1 0,0-1 0,-4 35 0,7-36 0,-1 1 0,-1 0 0,-1-1 0,0 0 0,-1 0 0,-2 0 0,-12 23 0,6-11 0,1 0 0,2 1 0,0 0 0,3 1 0,0 0 0,2 0 0,2 0 0,-1 34 0,3-52 0,0 0 0,0 1 0,-1-1 0,-1-1 0,-1 1 0,0 0 0,0-1 0,-1 0 0,-10 15 0,-1 7 0,13-29 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 0 0,-1 1 0,1-2 0,-1 1 0,0-1 0,0 0 0,-13 7 0,3-3 0,0-1 0,0-1 0,-33 8 0,42-12 0,0 1 0,1-1 0,0 1 0,-1 0 0,1 1 0,-6 4 0,7-5 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0-1 0,-10 2 0,-32 1 0,-1-2 0,1-2 0,-69-8 0,105 5 0,0-1 0,1-1 0,-1 1 0,1-2 0,0 1 0,1-2 0,-14-7 0,-33-16 0,-20 3-1365,54 20-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink86.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:15:00.639"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.3" units="cm"/>
-      <inkml:brushProperty name="height" value="0.6" units="cm"/>
-      <inkml:brushProperty name="color" value="#FFFC00"/>
-      <inkml:brushProperty name="tip" value="rectangle"/>
-      <inkml:brushProperty name="rasterOp" value="maskPen"/>
-      <inkml:brushProperty name="ignorePressure" value="1"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 240,'0'-4,"0"0,0 1,1-1,-1 0,1 0,0 1,0-1,0 0,1 1,-1-1,1 1,0-1,0 1,0 0,0 0,4-4,-2 3,1 0,0 0,0 1,0 0,1 0,-1 0,1 0,-1 1,12-3,34-9,-12 3,1-1,46-22,-62 22,1 1,0 1,1 2,0 0,0 1,0 2,1 1,49-2,1432 9,-1485-3</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink87.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:15:01.470"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.3" units="cm"/>
-      <inkml:brushProperty name="height" value="0.6" units="cm"/>
-      <inkml:brushProperty name="color" value="#FFFC00"/>
-      <inkml:brushProperty name="tip" value="rectangle"/>
-      <inkml:brushProperty name="rasterOp" value="maskPen"/>
-      <inkml:brushProperty name="ignorePressure" value="1"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 188,'8'-9,"-5"5,1 1,-1-1,1 1,-1 0,1 0,0 0,0 0,0 1,1-1,-1 1,1 0,-1 0,1 1,9-2,34-3,0 3,96 5,-37 2,-27-4,4 2,-1-5,88-12,-114 8,1 3,87 5,50-3,-160-2,63-17,-69 13,0 1,1 2,39-3,-50 7,0-2,0 0,-1-1,30-10,-29 7,2 1,-1 1,34-3,327 5,-188 6,293-3,-452 2,1 2,-1 2,48 13,-69-15,1 0,-1 2,15 7,-11-4</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink88.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:15:02.469"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.3" units="cm"/>
-      <inkml:brushProperty name="height" value="0.6" units="cm"/>
-      <inkml:brushProperty name="color" value="#FFFC00"/>
-      <inkml:brushProperty name="tip" value="rectangle"/>
-      <inkml:brushProperty name="rasterOp" value="maskPen"/>
-      <inkml:brushProperty name="ignorePressure" value="1"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 191,'0'-1,"1"0,-1 0,1 0,-1-1,1 1,-1 0,1 0,0 0,0 0,0 0,-1 0,1 0,0 1,0-1,0 0,0 0,1 1,-1-1,0 1,0-1,0 1,0-1,1 1,-1 0,0-1,0 1,3 0,40-5,-39 4,408-2,-212 6,513-3,-682-2,57-10,-53 7,42-3,75-5,13-1,-131 12,50-9,28-1,-74 11,-11 2,0-2,0 0,0-2,0-1,0-1,-1-1,38-15,-42 12,1 1,0 1,0 1,1 1,-1 1,28 0,157 5,-86 2,-60-4,-39-1,-1 1,1 1,0 1,-1 1,1 1,-1 1,0 1,30 11,-38-10,0-1,0 0,1-1,-1-1,1 0,18 0,97-3,-59-2,-49 2</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink89.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:15:03.600"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.3" units="cm"/>
-      <inkml:brushProperty name="height" value="0.6" units="cm"/>
-      <inkml:brushProperty name="color" value="#FFFC00"/>
-      <inkml:brushProperty name="tip" value="rectangle"/>
-      <inkml:brushProperty name="rasterOp" value="maskPen"/>
-      <inkml:brushProperty name="ignorePressure" value="1"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 362,'0'-1,"0"0,1-1,-1 1,1 0,-1 0,1 0,0 0,0 0,-1 0,1 0,0 0,0 0,0 0,0 0,0 1,0-1,0 0,0 1,0-1,0 1,1-1,-1 1,0-1,0 1,1 0,-1 0,2-1,41-4,-39 5,113-13,44-2,-8 18,128-6,-195-9,-56 6,48-2,-54 8,7 0,0-1,-1-2,1 0,54-15,-56 10,1 2,0 1,60-2,-44 4,54-9,-58 6,50-1,-45 7,1-3,-1-2,0-2,49-14,-58 12,44-3,-45 7,52-13,-41 7,88-9,-92 16,1-3,74-20,23-18,-118 37</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -14606,6 +15363,235 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:42.481"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">420 0 24575,'-6'0'0,"1"1"0,0-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 1 0,0 1 0,0-1 0,0 1 0,1 0 0,-1 0 0,1 0 0,0 0 0,-6 7 0,1 1 0,1 0 0,0 0 0,1 0 0,1 1 0,-11 25 0,8-20 0,0-1 0,-1 0 0,-1-1 0,-23 28 0,-24 33 0,28-21 0,-24 62 0,38-81 0,11-18 0,0 0 0,1 1 0,1-1 0,1 1 0,0 0 0,2 0 0,0 0 0,3 22 0,-1 14 0,-2-52 0,0 1 0,0-1 0,0 1 0,0-1 0,1 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0-1 0,4 4 0,-1-3 0,0-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,-1 0 0,1 0 0,-1-1 0,1 1 0,10-2 0,333-4 0,-342 5 0,-1-1 0,0 1 0,0-1 0,1-1 0,-1 1 0,0-1 0,0 0 0,0 0 0,-1-1 0,1 0 0,-1 0 0,1 0 0,4-4 0,5-5 0,-2-1 0,1 0 0,13-18 0,-20 20 0,-1 1 0,0-2 0,0 1 0,-1-1 0,-1 0 0,0 0 0,-1 0 0,0 0 0,0-1 0,0-15 0,-3 26 0,0 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,-3-1 0,-57-22 0,33 15 0,-4-5 0,-1 0 0,-1 3 0,0 1 0,-1 1 0,0 2 0,0 1 0,-45 0 0,57 6 0,-1-1 0,1-1 0,-46-9 0,2 1-1365,46 9-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink91.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:51.648"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 106 24575,'54'-20'0,"67"10"0,-81 8 0,53-8 0,109-17 0,-117 16 0,19-4 0,-101 14 0,48-8 0,-49 9 0,0-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,0 0 0,-1 0 0,1-1 0,-1 1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,2 2 0,-3-1 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,-3 3 0,-22 36 0,18-31 0,-1 6 0,0 1 0,1 0 0,0 1 0,2-1 0,0 1 0,1 0 0,-3 24 0,2-12 0,-13 44 0,4-14 0,13-51 0,-1 0 0,1 0 0,-2 0 0,1 0 0,-1 0 0,0-1 0,-1 1 0,0-1 0,0 0 0,-7 9 0,7-13 0,1 0 0,-1 1 0,1 0 0,0 0 0,0 0 0,-4 9 0,6-11 0,1 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,1 0 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 1 0,0-1 0,2 4 0,-2-3 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,-1 1 0,-1 2 0,-21 48 0,18-45 0,0 1 0,0-1 0,1 1 0,-3 13 0,-45 162-1365,49-166-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="449.47">31 314 24575,'894'0'0,"-877"-1"19,1-1 0,33-8 0,-11 1-1441,-18 6-5404</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink92.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:53.534"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">111 1 24575,'0'12'0,"2"0"0,-1 0 0,2 0 0,-1 0 0,2 0 0,0-1 0,0 1 0,1-1 0,1 0 0,0 0 0,0-1 0,2 0 0,8 11 0,-1 3 0,-1 1 0,-2 0 0,12 32 0,-10-23 0,7 36 0,-19-59 0,0 1 0,1-1 0,1 0 0,0 0 0,1 0 0,0-1 0,1 0 0,10 15 0,-3-11 0,-1 0 0,-1 0 0,-1 1 0,0 1 0,-1-1 0,0 1 0,8 25 0,-10-21 0,1-1 0,0 0 0,22 31 0,-22-37 0,1 0 0,-2 0 0,0 1 0,-1-1 0,-1 1 0,0 1 0,-1-1 0,4 26 0,-6-18 0,0 6 0,-2 0 0,-2 34 0,1-56 0,0-1 0,1 1 0,-2 0 0,1 0 0,-1 0 0,0-1 0,0 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,0-1 0,0 1 0,0-1 0,-8 7 0,6-8 0,0 1 0,0-2 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1-1 0,-1 1 0,0-1 0,-12 0 0,-79-4 0,49 0 0,13 4 0,22-1 0,-1 0 0,0 0 0,0-2 0,-24-4 0,34 5 0,0 0 0,1-1 0,-1 0 0,1 0 0,0 0 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,1-2 0,0 1 0,-1 0 0,1-1 0,1 1 0,-1-1 0,0 0 0,-2-6 0,-2-1 0,2 0 0,-1 0 0,1 0 0,1-1 0,0 1 0,1-1 0,0 0 0,1 0 0,1 0 0,0 0 0,0 0 0,2 0 0,-1 0 0,2 0 0,4-18 0,7-6 0,2 2 0,21-36 0,-10 22 0,-19 37 0,1 0 0,0 1 0,1 0 0,0 1 0,1-1 0,0 2 0,23-16 0,17-16 0,-24 16 0,-13 11 0,1 0 0,0 0 0,1 1 0,1 1 0,0 0 0,1 1 0,20-9 0,-18 10 0,1-2 0,-1 0 0,-1-1 0,20-16 0,-5 4 0,-25 19 0,0 0 0,0 1 0,1 0 0,-1 1 0,1 0 0,11-3 0,-12 4 0,0 0 0,0 0 0,0-1 0,-1 0 0,0-1 0,0 1 0,0-1 0,10-7 0,83-57 0,-99 67-40,1-1 0,-1 1 0,0-1 0,1 1-1,-1-1 1,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 0-1,-1 0 1,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0-1,0 0 1,-1 0 0,1 0 0,0 0 0,0 0 0,-1 1 0,0-1-1,1 0 1,-1 0 0,0 0 0,0 0 0,0 1 0,0-1-1,0 0 1,0 1 0,-2-3 0,-7-11-6786</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink93.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:14:54.983"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.035" units="cm"/>
+      <inkml:brushProperty name="height" value="0.035" units="cm"/>
+      <inkml:brushProperty name="color" value="#66CC00"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1901 74 24575,'-653'0'0,"626"-1"0,1-2 0,-31-6 0,29 4 0,1 1 0,-28-1 0,-370 6 0,409 1 0,1 1 0,-1 0 0,1 1 0,0 1 0,0 0 0,0 1 0,1 1 0,-25 15 0,-6 1 0,35-17 0,0 1 0,1 0 0,-1 0 0,1 0 0,1 1 0,0 1 0,0 0 0,0 0 0,1 0 0,-7 13 0,-33 38 0,39-51 0,1 0 0,1 0 0,0 1 0,0 0 0,1 0 0,0 0 0,1 0 0,0 1 0,0 0 0,1 0 0,1 0 0,-2 12 0,0 17 0,3 82 0,2-84 0,-2-34 0,1 0 0,1 0 0,-1 1 0,0-1 0,1 0 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,0 0 0,0-1 0,1 1 0,-1-1 0,1 0 0,3 4 0,1-2 0,0-1 0,0 1 0,1-1 0,0-1 0,-1 1 0,1-1 0,16 4 0,10 1 0,0-2 0,0 0 0,65 0 0,105-13 0,-178 6 0,0-3 0,29-6 0,-46 8 0,1-1 0,-1 0 0,0 0 0,0-1 0,0-1 0,-1 1 0,1-2 0,-1 1 0,8-7 0,59-44 0,-17 14 0,-50 36 0,6-4 0,-1-2 0,0 0 0,16-17 0,-25 23 0,1-1 0,-1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,-1-1 0,0 1 0,0 0 0,1-12 0,20-167 0,-11 112 0,-7 48 0,-1 0 0,0-33 0,-3 44 0,-1 10 0,1 0 0,-1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,-3-7 0,4 11 0,0 1 0,-1 0 0,1-1 0,0 1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 0 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 1 0,0-1 0,-1 0 0,1 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 0 0,-1 2 0,-18 25 0,16-22 0,-87 145 0,81-132 0,1 0 0,1 1 0,0 0 0,2 1 0,0-1 0,-4 35 0,7-36 0,-1 1 0,-1 0 0,-1-1 0,0 0 0,-1 0 0,-2 0 0,-12 23 0,6-11 0,1 0 0,2 1 0,0 0 0,3 1 0,0 0 0,2 0 0,2 0 0,-1 34 0,3-52 0,0 0 0,0 1 0,-1-1 0,-1-1 0,-1 1 0,0 0 0,0-1 0,-1 0 0,-10 15 0,-1 7 0,13-29 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 0 0,-1 1 0,1-2 0,-1 1 0,0-1 0,0 0 0,-13 7 0,3-3 0,0-1 0,0-1 0,-33 8 0,42-12 0,0 1 0,1-1 0,0 1 0,-1 0 0,1 1 0,-6 4 0,7-5 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,0-1 0,-10 2 0,-32 1 0,-1-2 0,1-2 0,-69-8 0,105 5 0,0-1 0,1-1 0,-1 1 0,1-2 0,0 1 0,1-2 0,-14-7 0,-33-16 0,-20 3-1365,54 20-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink94.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:15:00.639"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.3" units="cm"/>
+      <inkml:brushProperty name="height" value="0.6" units="cm"/>
+      <inkml:brushProperty name="color" value="#FFFC00"/>
+      <inkml:brushProperty name="tip" value="rectangle"/>
+      <inkml:brushProperty name="rasterOp" value="maskPen"/>
+      <inkml:brushProperty name="ignorePressure" value="1"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 240,'0'-4,"0"0,0 1,1-1,-1 0,1 0,0 1,0-1,0 0,1 1,-1-1,1 1,0-1,0 1,0 0,0 0,4-4,-2 3,1 0,0 0,0 1,0 0,1 0,-1 0,1 0,-1 1,12-3,34-9,-12 3,1-1,46-22,-62 22,1 1,0 1,1 2,0 0,0 1,0 2,1 1,49-2,1432 9,-1485-3</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink95.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:15:01.470"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.3" units="cm"/>
+      <inkml:brushProperty name="height" value="0.6" units="cm"/>
+      <inkml:brushProperty name="color" value="#FFFC00"/>
+      <inkml:brushProperty name="tip" value="rectangle"/>
+      <inkml:brushProperty name="rasterOp" value="maskPen"/>
+      <inkml:brushProperty name="ignorePressure" value="1"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 188,'8'-9,"-5"5,1 1,-1-1,1 1,-1 0,1 0,0 0,0 0,0 1,1-1,-1 1,1 0,-1 0,1 1,9-2,34-3,0 3,96 5,-37 2,-27-4,4 2,-1-5,88-12,-114 8,1 3,87 5,50-3,-160-2,63-17,-69 13,0 1,1 2,39-3,-50 7,0-2,0 0,-1-1,30-10,-29 7,2 1,-1 1,34-3,327 5,-188 6,293-3,-452 2,1 2,-1 2,48 13,-69-15,1 0,-1 2,15 7,-11-4</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink96.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:15:02.469"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.3" units="cm"/>
+      <inkml:brushProperty name="height" value="0.6" units="cm"/>
+      <inkml:brushProperty name="color" value="#FFFC00"/>
+      <inkml:brushProperty name="tip" value="rectangle"/>
+      <inkml:brushProperty name="rasterOp" value="maskPen"/>
+      <inkml:brushProperty name="ignorePressure" value="1"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 191,'0'-1,"1"0,-1 0,1 0,-1-1,1 1,-1 0,1 0,0 0,0 0,0 0,-1 0,1 0,0 1,0-1,0 0,0 0,1 1,-1-1,0 1,0-1,0 1,0-1,1 1,-1 0,0-1,0 1,3 0,40-5,-39 4,408-2,-212 6,513-3,-682-2,57-10,-53 7,42-3,75-5,13-1,-131 12,50-9,28-1,-74 11,-11 2,0-2,0 0,0-2,0-1,0-1,-1-1,38-15,-42 12,1 1,0 1,0 1,1 1,-1 1,28 0,157 5,-86 2,-60-4,-39-1,-1 1,1 1,0 1,-1 1,1 1,-1 1,0 1,30 11,-38-10,0-1,0 0,1-1,-1-1,1 0,18 0,97-3,-59-2,-49 2</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink97.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:15:03.600"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.3" units="cm"/>
+      <inkml:brushProperty name="height" value="0.6" units="cm"/>
+      <inkml:brushProperty name="color" value="#FFFC00"/>
+      <inkml:brushProperty name="tip" value="rectangle"/>
+      <inkml:brushProperty name="rasterOp" value="maskPen"/>
+      <inkml:brushProperty name="ignorePressure" value="1"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 362,'0'-1,"0"0,1-1,-1 1,1 0,-1 0,1 0,0 0,0 0,-1 0,1 0,0 0,0 0,0 0,0 0,0 1,0-1,0 0,0 1,0-1,0 1,1-1,-1 1,0-1,0 1,1 0,-1 0,2-1,41-4,-39 5,113-13,44-2,-8 18,128-6,-195-9,-56 6,48-2,-54 8,7 0,0-1,-1-2,1 0,54-15,-56 10,1 2,0 1,60-2,-44 4,54-9,-58 6,50-1,-45 7,1-3,-1-2,0-2,49-14,-58 12,44-3,-45 7,52-13,-41 7,88-9,-92 16,1-3,74-20,23-18,-118 37</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink98.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:22.767"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
@@ -14618,7 +15604,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink91.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink99.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -14643,235 +15629,6 @@
     </inkml:brush>
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">1 265 24575,'0'-6'0,"0"0"0,1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,0-1 0,0 0 0,0 1 0,1-1 0,0 1 0,0 0 0,0 0 0,5-5 0,0 1 0,0 1 0,1 0 0,0 1 0,0 0 0,1 0 0,15-8 0,14-15 0,-34 25 0,-1 1 0,2 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1 0 0,11-4 0,-6 4 0,24-8 0,1 1 0,0 2 0,44-4 0,-73 11 0,1 1 0,0-1 0,0 1 0,0 0 0,0 1 0,0 0 0,-1 0 0,1 0 0,0 1 0,-1 1 0,1-1 0,-1 1 0,0 0 0,0 1 0,0-1 0,0 1 0,0 1 0,-1-1 0,0 1 0,0 0 0,8 9 0,-13-11 0,1 0 0,-1 0 0,0 0 0,1 0 0,-2 0 0,1 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,0 1 0,-3 3 0,-2 2 0,-1 0 0,1 0 0,-1-1 0,0 0 0,-1 0 0,0-1 0,-16 9 0,-18 2 0,36-15 0,0 0 0,0 1 0,0 0 0,0 0 0,1 1 0,-1-1 0,1 1 0,0 1 0,-7 6 0,-3 2 0,0 0 0,-33 20 0,30-22 0,2 1 0,-31 27 0,34-26 0,0 0 0,2 1 0,0 0 0,0 1 0,2 0 0,0 1 0,0 0 0,2 1 0,0 0 0,1 0 0,1 1 0,-6 24 0,0 12 0,6-32 0,1 1 0,1 0 0,-1 45 0,5-62 0,0 0 0,1 0 0,-1 0 0,1 0 0,1-1 0,-1 1 0,1 0 0,0-1 0,1 1 0,-1-1 0,1 0 0,0 1 0,1-1 0,-1-1 0,1 1 0,0 0 0,0-1 0,0 0 0,1 0 0,5 4 0,8 2 0,-1-1 0,2 0 0,-1-2 0,1 0 0,0-1 0,1 0 0,35 4 0,38 11 0,-43-10-38,0-3 0,1-1 0,1-3 0,-1-2 0,62-5-1,-21 2-1097,-64 1-5690</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink92.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:54.858"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">332 96 24575,'1'-1'0,"0"-1"0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,4-1 0,13-7 0,-11 3 0,1-1 0,0 0 0,0 0 0,1 1 0,0 0 0,0 1 0,0 0 0,1 0 0,-1 1 0,19-3 0,22 1 0,0 2 0,0 3 0,60 6 0,-108-6 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1 0 0,3 3 0,-3-4 0,-1 1 0,0 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-2 4 0,-1 3 0,-1 0 0,-1-1 0,0 1 0,0-1 0,-1 0 0,0 0 0,0-1 0,-14 14 0,3-8 0,0 0 0,-1-1 0,0 0 0,-37 16 0,5-2 0,4 5 0,38-24 0,0-1 0,-1 0 0,0-1 0,0 0 0,-19 8 0,9-6 0,0 0 0,1 1 0,0 1 0,0 0 0,1 2 0,-27 20 0,-11 5 0,42-29 0,0 1 0,1 0 0,-16 14 0,16-10 0,-1-1 0,-1 0 0,0 0 0,0-1 0,-1-1 0,-1 0 0,-16 6 0,26-12 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,1 1 0,0-1 0,0 1 0,0 0 0,1 0 0,0 0 0,-5 7 0,8-10 0,0-1 0,0 1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,2 0 0,-1 0 0,0 0 0,0 0 0,1 0 0,0 3 0,0-3 0,1 1 0,-1-1 0,1 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,1-1 0,0 0 0,2 2 0,26 7 0,0-1 0,0-1 0,0-2 0,1-1 0,0-1 0,0-1 0,44-3 0,81 10 0,76 32 0,-193-38 0,1-1 0,0-2 0,40-4 0,-43 0 0,0 2 0,0 2 0,59 8 0,-93-8 0,1-1 0,-1 1 0,1 1 0,-1-1 0,1 0 0,-1 1 0,0 0 0,0 0 0,0 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,0 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,0-1 0,0 0 0,0 1 0,-1-1 0,0 0 0,0 1 0,0-1 0,-1 0 0,1 1 0,-1-1 0,0 0 0,-3 8 0,2-8 0,0-1 0,0 0 0,0 0 0,-1-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,1-1 0,-2 0 0,1 0 0,0 0 0,0 0 0,-1 0 0,-6 1 0,-60 16 0,48-15 0,-30 7 0,30-8 0,1 1 0,0 1 0,-36 14 0,17 3 0,30-16 0,1-1 0,-1 0 0,0 0 0,-16 5 0,-44 15 78,51-17-559,-1 0 0,-32 7 0,29-11-6345</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink93.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:58.689"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1221 1 24575,'-13'0'0,"0"0"0,-1 2 0,1 0 0,0 0 0,0 1 0,0 1 0,1 0 0,-1 0 0,1 2 0,0-1 0,0 2 0,1-1 0,0 1 0,0 1 0,0 0 0,1 1 0,-10 11 0,-1 3 0,1 0 0,1 2 0,1 0 0,2 1 0,-16 31 0,-8 19 0,30-61 0,0 1 0,2 0 0,0 1 0,1 0 0,0 0 0,2 1 0,0 0 0,1 0 0,-3 29 0,3-7 0,-1 0 0,-2-1 0,-14 45 0,11-42 0,1 7 0,3 0 0,2 0 0,2 0 0,7 68 0,-2 0 0,-2-106 0,0 0 0,1 1 0,0-1 0,1-1 0,0 1 0,1 0 0,0-1 0,0 1 0,1-1 0,1-1 0,0 1 0,0-1 0,1 0 0,0 0 0,1 0 0,12 10 0,58 32 0,-70-46 0,0 1 0,1-1 0,-1 0 0,1-1 0,0 1 0,1-2 0,-1 0 0,1 0 0,-1 0 0,1-1 0,0-1 0,0 0 0,0 0 0,0 0 0,12-2 0,-13 0 0,-1 1 0,1-1 0,0 0 0,-1-1 0,1 0 0,-1-1 0,0 1 0,0-1 0,0-1 0,0 0 0,0 0 0,-1 0 0,1-1 0,-1 0 0,0-1 0,-1 1 0,8-10 0,25-30 0,-31 37 0,0 0 0,0-1 0,-1 0 0,0-1 0,-1 0 0,0 0 0,0 0 0,-1-1 0,6-17 0,-9 17 0,1 0 0,1 0 0,0 0 0,0 0 0,1 1 0,0 0 0,1 0 0,0 0 0,1 1 0,0 0 0,0 0 0,1 0 0,15-12 0,-14 13 0,-1 0 0,0-1 0,-1-1 0,0 1 0,0-1 0,-1 0 0,0-1 0,0 1 0,-2-1 0,1 0 0,-1-1 0,-1 1 0,3-13 0,-2-1 0,0 0 0,-2 0 0,-1 0 0,0 0 0,-5-30 0,3 51 0,0 0 0,0 0 0,0 0 0,-1 0 0,0 0 0,0 0 0,0 1 0,0-1 0,0 1 0,-1-1 0,0 1 0,1 0 0,-1 0 0,0 0 0,-1 0 0,1 1 0,-6-5 0,3 3 0,0 0 0,1-1 0,0 0 0,0-1 0,-6-7 0,3 2 0,-1 1 0,0 1 0,0-1 0,-1 1 0,0 1 0,-15-10 0,11 8 0,1 0 0,0-1 0,-13-14 0,22 20 0,-1 1 0,0 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 1 0,0-1 0,0 1 0,0 0 0,0 1 0,-1-1 0,1 1 0,-8 0 0,-15-1 0,0 1 0,-35 4 0,13 0 0,30-4 0,0 2 0,0 0 0,1 2 0,-1 0 0,0 1 0,1 1 0,-27 10 0,21-5 0,-44 9 0,55-16 0,0 1 0,0 0 0,0 1 0,0 0 0,1 1 0,0 1 0,0 0 0,-21 15 0,19-9 0,-1-1 0,0-1 0,-1-1 0,-27 11 0,25-9 0,0 0 0,0 1 0,2 1 0,-27 25 0,13-11 0,-78 74 0,100-92 17,0 1-1,0 0 1,0 0 0,2 1-1,-1 0 1,2 1-1,-11 21 1,10-17-392,-2 0 1,0 0-1,-17 20 1,15-23-6452</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink94.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:57.160"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">103 3 24575,'1'69'0,"-3"80"0,0-137 0,-1 0 0,0 0 0,-1 0 0,0 0 0,-1-1 0,-7 13 0,-17 44 0,21-42 0,-2 8 0,-9 53 0,18-78 0,0 1 0,0-1 0,1 1 0,1-1 0,-1 1 0,1 0 0,1-1 0,0 0 0,1 1 0,5 13 0,-4-17 0,0-1 0,1 1 0,-1-1 0,1 0 0,1 0 0,-1 0 0,1-1 0,0 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,1-2 0,11 4 0,33 19 0,-18-7 0,0-1 0,1-2 0,1-1 0,36 10 0,-44-15 0,-21-7 0,-1 0 0,0 1 0,0 0 0,0 0 0,0 0 0,0 0 0,-1 1 0,1 0 0,-1 0 0,0 0 0,4 6 0,36 58 0,-23-32 0,-13-21 0,0 0 0,-1 0 0,-1 1 0,6 26 0,-6-22 0,0-1 0,15 32 0,-11-29 0,-1 0 0,-1 0 0,9 38 0,-16-57 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,-1 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,-1 0 0,1 0 0,-1-1 0,0 1 0,-2 3 0,0-2 0,0-1 0,0 0 0,-1 0 0,1 0 0,-1 0 0,1-1 0,-1 1 0,0-1 0,0 0 0,0-1 0,-8 3 0,-13 0 0,1-1 0,-1-1 0,1-1 0,-30-2 0,46 1 0,-33-1 0,29 2 0,0 0 0,1-2 0,-1 1 0,0-2 0,0 1 0,0-2 0,1 1 0,0-2 0,-18-6 0,11 0 40,1 0 0,-23-17 0,35 22-175,0 1 0,1-1 0,0-1 0,0 1 0,0-1 0,1 0 0,0 0 0,0 0 0,1 0 0,-4-9 0,-1-6-6691</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="419.51">48 34 24575,'5'-3'0,"-1"0"0,1 0 0,0 0 0,0 0 0,0 1 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 1 0,-1 0 0,9-1 0,76-1 0,-61 3 0,50-2 0,239 6 0,-306-2 0,0 1 0,0 0 0,0 0 0,-1 1 0,0 1 0,16 7 0,41 16 0,-55-24 30,0 0-1,-1 2 0,19 9 1,11 6-1513,-22-14-5343</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink95.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:24:55.603"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">325 0 24575,'0'9'0,"-1"1"0,-1-1 0,1 0 0,-1 0 0,-1 0 0,1 0 0,-1-1 0,-1 1 0,0-1 0,-7 12 0,-7 9 0,-34 41 0,34-50 0,2 2 0,-25 44 0,32-47 0,2 1 0,-7 25 0,-13 36 0,17-57 0,-11 45 0,15-48 0,0 0 0,-2-1 0,-11 26 0,16-40 0,0 0 0,0 0 0,1 1 0,0 0 0,0-1 0,1 1 0,-1 0 0,1 0 0,1 0 0,-1 0 0,1 0 0,1 0 0,-1 0 0,1 0 0,2 8 0,-2-10 0,0-1 0,1 0 0,-1 0 0,1 0 0,0 0 0,0 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,1 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0-1 0,1 1 0,0-1 0,-1 0 0,1 0 0,0-1 0,0 1 0,0-1 0,8 2 0,25 1 0,1-1 0,-1-2 0,55-6 0,5 1 0,-59 5 0,-27 0 0,1 0 0,-1-1 0,0 0 0,0-1 0,1-1 0,-1 1 0,0-2 0,0 0 0,-1 0 0,12-5 0,45-32-1365,-50 26-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="446.47">520 535 24575,'-1'34'0,"-3"1"0,-7 37 0,5-37 0,-4 70 0,10-103 0,0 35 0,-1 0 0,-2-1 0,-10 53 0,7-50 0,1 1 0,2 1 0,2-1 0,4 50 0,-1-33 0,-4 58 0,-15-40-1365,11-54-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink96.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:25:03.802"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">692 1 24575,'-65'-1'0,"-77"3"0,137-1 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 1 0,1 0 0,-1 0 0,1 0 0,0 1 0,0-1 0,0 1 0,0 0 0,0 0 0,1 1 0,-5 4 0,-3 6 0,0 1 0,-17 29 0,-15 21 0,32-52 0,1 0 0,0 1 0,0 1 0,2-1 0,-1 2 0,2-1 0,0 1 0,-8 28 0,9-18 0,1 1 0,1 0 0,1 0 0,1 49 0,2 33 0,3 89 0,-2-190 0,0 0 0,1-1 0,0 1 0,0 0 0,1 0 0,0-1 0,0 0 0,1 1 0,0-1 0,0-1 0,10 13 0,3 0 0,1-1 0,27 22 0,-28-25 0,-9-7 0,0 0 0,-1 0 0,11 17 0,-14-18 0,1-1 0,0 1 0,0-1 0,0 0 0,1 0 0,0-1 0,0 1 0,0-1 0,9 4 0,1 1 0,-1 0 0,22 20 0,-6-5 0,-31-25 0,1 0 0,-1 0 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 0 0,0 1 0,1-1 0,-1 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0 0 0,-16 5 0,-32-5 0,42-1 0,-10-2 0,0 0 0,0-2 0,0 0 0,0-1 0,1 0 0,-1-1 0,1-1 0,-19-12 0,-29-12 0,-121-37 0,178 66 0,1-1 0,0 1 0,1-1 0,-1-1 0,0 1 0,1-1 0,-1 0 0,1 0 0,0 0 0,1 0 0,-1-1 0,1 0 0,0 1 0,0-2 0,0 1 0,0 0 0,1 0 0,0-1 0,-1-5 0,0 3 0,1 0 0,-1 0 0,2 0 0,-1 0 0,1 0 0,1-1 0,-1 1 0,1 0 0,1 0 0,0-1 0,0 1 0,4-16 0,-4 21 0,1-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,6-3 0,3 1 0,-1 0 0,1 1 0,22-3 0,-25 4 0,1 1 0,0-1 0,0-1 0,-1 0 0,1 0 0,10-6 0,42-28 0,87-39 0,-137 70 0,-1 0 0,0-1 0,15-11 0,-18 11 0,1 1 0,0 0 0,0 1 0,0 0 0,20-7 0,-18 9 0,-1 0 0,1-1 0,-1 0 0,0 0 0,-1-1 0,1 0 0,-1-1 0,0 0 0,0 0 0,11-12 0,0-2 0,-12 14 0,-1-1 0,0 0 0,0-1 0,-1 1 0,0-1 0,8-14 0,-13 19 0,0 0 0,0-1 0,0 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,-1 1 0,1 0 0,-1 0 0,1 0 0,-1 0 0,0 1 0,-3-4 0,-27-32-1365,18 22-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink97.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:25:02.154"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.035" units="cm"/>
-      <inkml:brushProperty name="height" value="0.035" units="cm"/>
-      <inkml:brushProperty name="color" value="#66CC00"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">567 1 24575,'-1'0'0,"0"0"0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 1 0,1 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,0-1 0,1 1 0,-1 0 0,0 0 0,1-1 0,0 2 0,0 1 0,1 1 0,0 0 0,-1-1 0,1 1 0,1-1 0,-1 0 0,0 0 0,1 0 0,3 3 0,0-2 0,1 0 0,0 0 0,-1-1 0,1 0 0,1 0 0,-1 0 0,0-1 0,1-1 0,13 3 0,73-1 0,-76-4 0,0 1 0,0 0 0,0 2 0,34 6 0,-52-8 0,1 0 0,-1 0 0,1 0 0,-1 0 0,1 0 0,0 1 0,-1-1 0,1 0 0,-1 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 1 0,1-1 0,-1 1 0,1-1 0,-1 0 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,1-1 0,-1 1 0,0-1 0,0 1 0,0-1 0,1 1 0,-1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 1 0,-1-1 0,1 1 0,0 0 0,-22 25 0,-38 16 0,56-39 0,-8 3 0,0 1 0,1 0 0,0 1 0,0 0 0,1 0 0,0 1 0,0 1 0,-11 14 0,4-3 0,-34 34 0,32-36 0,-33 41 0,14-8 0,-3-3 0,-81 78 0,109-114 0,2 1 0,0 0 0,0 1 0,1 0 0,1 1 0,1 0 0,0 0 0,1 1 0,1 0 0,-4 21 0,5-25 0,0 0 0,-1 0 0,0-1 0,-1 0 0,-16 22 0,-10 18 0,-3-4 0,29-40 0,0 1 0,0 0 0,-9 16 0,9-11-273,0-1 0,1 1 0,1 0 0,-5 21 0,6-12-6553</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="365.01">0 1004 24575,'0'-2'0,"1"1"0,0-1 0,-1 1 0,1 0 0,0-1 0,-1 1 0,1 0 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,4 1 0,48-6 0,-47 6 0,195 0 0,21-2 0,-195-1 0,1-1 0,-1-1 0,0-2 0,-1-1 0,0 0 0,0-2 0,-1-1 0,33-19 0,-44 23 0,0 1 0,0 1 0,0 0 0,1 1 0,0 0 0,0 1 0,19-1 0,-25 2 0,-3 1-124,-1 0 0,1-1 0,0 0 0,-1 0 0,0 0 0,1-1-1,-1 0 1,0 0 0,0 0 0,6-6 0,4-3-6702</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink98.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:25:10.409"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.3" units="cm"/>
-      <inkml:brushProperty name="height" value="0.6" units="cm"/>
-      <inkml:brushProperty name="color" value="#FFFC00"/>
-      <inkml:brushProperty name="tip" value="rectangle"/>
-      <inkml:brushProperty name="rasterOp" value="maskPen"/>
-      <inkml:brushProperty name="ignorePressure" value="1"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1,'8'0,"1"0,0 0,0 1,0 0,0 1,-1-1,1 2,-1-1,1 1,-1 1,0-1,0 1,0 1,-1 0,7 5,-3-3,-1 0,1-1,0 0,1-1,-1 0,1-1,0 0,0-1,0-1,13 2,33 8,25 2,32 3,-77-10,75 4,-102-12,1 1,0 1,-1 0,1 1,0 0,-1 1,0 0,0 1,0 0,11 6,-3-2,-1-2,1-1,0 0,0-1,0-1,0-1,36 0,54 8,22 4,-71-9,-49-3,-1 0,0 1,0 0,0 1,0 0,12 7,-11-5,0-1,0 0,1-1,18 5,74 0,-74-8,1 2,31 6,-24-2,1-2,-1-2,1-1,74-7,-108 4,0 0,-1 0,1-1,0 1,0-1,-1 0,1-1,-1 1,0-1,0 1,0-1,5-5,5-4</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink99.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-10-10T07:25:11.398"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.3" units="cm"/>
-      <inkml:brushProperty name="height" value="0.6" units="cm"/>
-      <inkml:brushProperty name="color" value="#FFFC00"/>
-      <inkml:brushProperty name="tip" value="rectangle"/>
-      <inkml:brushProperty name="rasterOp" value="maskPen"/>
-      <inkml:brushProperty name="ignorePressure" value="1"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1,'1807'0,"-1798"0,1 1,0 0,-1 1,1 0,-1 0,1 1,-1 0,0 1,0 0,-1 1,1-1,-1 2,11 7,-13-9,12 6,0-2,1-1,0 0,0-1,1-1,34 4,-11-1,-6-3,0-1,0-2,44-3,-46-1,1 2,-1 2,60 10,-58-5,1-1,73 2,-84-8</inkml:trace>
 </inkml:ink>
 </file>
 

</xml_diff>